<commit_message>
feat(query): semester credit totals with the 9-22 limit, taking a course together with its prerequisite, effect of a stated low GPA; treat lowercase it/bit as English words; hard/challenge unseen round 7; tester 661 rows
</commit_message>
<xml_diff>
--- a/docs/tester.xlsx
+++ b/docs/tester.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O634"/>
+  <dimension ref="A1:O662"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10" customWidth="1" style="36" min="1" max="1"/>
@@ -756,7 +756,7 @@
       </c>
       <c r="N2" s="13" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.03s</t>
         </is>
       </c>
       <c r="O2" s="21" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="N7" s="25" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.04s</t>
         </is>
       </c>
       <c r="O7" s="21" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="N9" s="25" t="inlineStr">
         <is>
-          <t>0.73s</t>
+          <t>0.62s</t>
         </is>
       </c>
       <c r="O9" s="21" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="N10" s="13" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O10" s="21" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="N11" s="25" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O11" s="21" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="N12" s="13" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="O12" s="21" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="N13" s="25" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.35s</t>
         </is>
       </c>
       <c r="O13" s="21" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="N14" s="13" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="O14" s="21" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="N15" s="25" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="O15" s="21" t="inlineStr">
@@ -2395,7 +2395,7 @@
       <c r="G21" s="34" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาสามารถเรียนวิชาฐานข้อมูลในปีที่ 4 ได้ เนื่องจากหลักสูตรมีวิชาบังคับที่เกี่ยวข้องกับฐานข้อมูล เช่น 06026246 ระบบฐานข้อมูลแบบกระจาย และ 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 ซึ่งจัดสอนในภาคการศึกษาที่ 1 ปีที่ 4 โดยมีวิชาบังคับก่อนอย่าง 06066300 แนวคิดระบบฐานข้อมูล (ปีที่ 2 ภาคการศึกษาที่ 1) ที่เป็นพื้นฐานสำคัญ</t>
+นักศึกษาสามารถเรียนวิชาที่เกี่ยวข้องกับฐานข้อมูลในปีที่ 4 ได้ เนื่องจากมีวิชาบังคับก่อนหน้า เช่น 06066300 แนวคิดระบบฐานข้อมูล (ปี 2 ภาค 1) และ 06026212 การสร้างคลังข้อมูล (ปี 3 ภาค 1) ซึ่งเป็นพื้นฐานจำเป็น วิชาที่เกี่ยวข้องในปี 4 ได้แก่ 06026246 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 และ 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 2 ที่จัดสอนในภาคการศึกษาที่ 1 ปีที่ 4 ประเภทวิชาบังคับในกลุ่มวิชาเลือกเฉพาะแขนง ตามหลักสูตร DSBA 2565</t>
         </is>
       </c>
       <c r="H21" s="34" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="K21" s="19" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L21" s="21" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="N21" s="13" t="inlineStr">
         <is>
-          <t>1.51s</t>
+          <t>2.88s</t>
         </is>
       </c>
       <c r="O21" s="21" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="N23" s="13" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.15s</t>
         </is>
       </c>
       <c r="O23" s="21" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="N24" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O24" s="21" t="inlineStr">
@@ -2801,15 +2801,11 @@
       </c>
       <c r="G25" s="34" t="inlineStr">
         <is>
-          <t>ใช่ หลักสูตรวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปีที่ 3 มีการเลือกแขนง (หรือที่เรียกว่า "กลุ่มวิชา") ซึ่งแบ่งออกเป็น 3 กลุ่ม ดังนี้:
-- วิชาเลือกกลุ่มวิทยาการข้อมูล 1 (ELECTIVE IN DATA SCIENCE 1) – 3 (3-0-6) หรือ 3 (2-2-5) [3]
-- วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 1 (ELECTIVE IN STATISTICAL ANALYSIS 1) – 3 (3-0-6) หรือ 3 (2-2-5) [3]
-- วิชาเลือกกลุ่มวิศวกรรมข้อมูล 1 (ELECTIVE IN DATA ENGINEERING 1) – 3 (3-0-6) หรือ 3 (2-2-5) [3]
-ในภาคการศึกษาที่ 2 ปีที่ 3 ยังมีการเลือกแขนงในลักษณะเดียวกัน ได้แก่:
-- วิชาเลือกกลุ่มวิทยาการข้อมูล 3 (ELECTIVE IN DATA SCIENCE 3) – 3 (3-0-6) หรือ 3 (2-2-5) [4]
-- วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 3 (ELECTIVE IN STATISTICAL ANALYTICS 3) – 3 (3-0-6) หรือ 3 (2-2-5) [4]
-- วิชาเลือกกลุ่มวิศวกรรมข้อมูล 3 (ELECTIVE IN DATA ENGINEERING 3) – 3 (3-0-6) หรือ 3 (2-2-5) [4]
-ดังนั้น แขนงที่สามารถเลือกได้คือ วิทยาการข้อมูล, การวิเคราะห์เชิงสถิติ, และวิศวกรรมข้อมูล [3][4]</t>
+          <t>ใช่ หลักสูตรวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปีที่ 3 มีการเลือกแขนง (หรือที่เรียกว่า "กลุ่มวิชา") ให้เลือก โดยมี 3 แขนง ดังนี้:
+- กลุ่มวิทยาการข้อมูล (Data Science)  
+- กลุ่มการวิเคราะห์เชิงสถิติ (Statistical Analytics)  
+- กลุ่มวิศวกรรมข้อมูล (Data Engineering)  
+[3][4][6]</t>
         </is>
       </c>
       <c r="H25" s="34" t="inlineStr">
@@ -2842,7 +2838,7 @@
       </c>
       <c r="N25" s="13" t="inlineStr">
         <is>
-          <t>4.29s</t>
+          <t>1.64s</t>
         </is>
       </c>
       <c r="O25" s="21" t="inlineStr">
@@ -2884,9 +2880,9 @@
       </c>
       <c r="G26" s="34" t="inlineStr">
         <is>
-          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวม 129 หน่วยกิต ลดลง 1 หน่วยกิตจาก IT 2560 ที่มี 130 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูลแทนการเลือกแขนงวิชาเดิม
-2. หลักสูตร IT 2565 ลดหน่วยกิตกลุ่มวิชาเฉพาะด้านจาก 46 หน่วยกิต (IT 2560) เป็น 57 หน่วยกิต แต่เพิ่มหน่วยกิตกลุ่มวิชาเลือกทางเทคโนโลยีสารสนเทศจาก 6 เป็น 9 หน่วยกิต โดยจัดเป็น 3 โมดูลอาชีพ (M1: Full-Stack Web Developer, M2: Network/System Engineer, M3: Game Developer) ซึ่งนักศึกษาสามารถเลือกเรียนได้ตามความสนใจ โดยไม่จำเป็นต้องเลือกครบ 3 โมดูล
-3. อ้างข้อมูลจาก: หน่วยกิตรวม (มคอ.2 IT 2560 หน้า 18, IT 2565 หน้า 6), โครงสร้างหลักสูตร (มคอ.2 IT 2565 หน้า 371, 374, 376, 378), กลุ่มวิชาเลือก (IT 2565 หน้า 378), กลุ่มวิชาเฉพาะด้าน (IT 2565 หน้า 374), กลุ่มวิชาบังคับเฉพาะสาขา (IT 2565 หน้า 376), ประเภทวิชา (บังคับ/เลือก) และการจัดกลุ่มโมดูล (IT 2565 หน้า 370, 378)</t>
+          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวมน้อยกว่า IT 2560 อยู่ 1 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูลแทนการเลือกแขนงวิชาเดิม
+2. หลักสูตร IT 2560 มีหน่วยกิตรวม 130 หน่วยกิต (มคอ.2 IT 2560 หน้า 18) ขณะที่ IT 2565 มี 129 หน่วยกิต (มคอ.2 IT 2565 หน้า 6) ลดลง 1 หน่วยกิต ซึ่งสะท้อนจากการปรับโครงสร้างกลุ่มวิชาเฉพาะด้านและวิชาเลือก โดยเฉพาะการเปลี่ยนจาก "แขนงวิชา" มาเป็น "โมดูลอาชีพ" 3 โมดูล (M1-M3) ที่มีความยืดหยุ่นในการเลือกวิชา และลดหน่วยกิตในกลุ่มวิชาบังคับเฉพาะแขนงจาก 30 เป็น 15 หน่วยกิต (ข้อมูลจาก [3], [4], [8])
+3. อ้างข้อมูลจากหลักฐาน: หน่วยกิตรวม (IT 2560 vs IT 2565), ประเภทวิชา (บังคับ/เลือก), ภาค/ปีที่เปิดสอน (IT 2560 เริ่มภาค 1/2560, IT 2565 เริ่มภาค 1/2565), โครงสร้างแขนงวิชา (เปลี่ยนจาก "แขนงวิชา" เป็น "โมดูลอาชีพ")</t>
         </is>
       </c>
       <c r="H26" s="34" t="inlineStr">
@@ -2919,7 +2915,7 @@
       </c>
       <c r="N26" s="13" t="inlineStr">
         <is>
-          <t>4.95s</t>
+          <t>4.90s</t>
         </is>
       </c>
       <c r="O26" s="21" t="inlineStr">
@@ -3071,7 +3067,7 @@
       <c r="M28" s="34" t="n"/>
       <c r="N28" s="13" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.44s</t>
         </is>
       </c>
       <c r="O28" s="21" t="inlineStr">
@@ -3147,7 +3143,7 @@
       </c>
       <c r="N29" s="25" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.16s</t>
         </is>
       </c>
       <c r="O29" s="21" t="inlineStr">
@@ -3488,7 +3484,7 @@
       </c>
       <c r="N33" s="25" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.30s</t>
         </is>
       </c>
       <c r="O33" s="21" t="inlineStr">
@@ -3636,7 +3632,7 @@
       <c r="M35" s="35" t="n"/>
       <c r="N35" s="25" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.52s</t>
         </is>
       </c>
       <c r="O35" s="21" t="inlineStr">
@@ -3804,7 +3800,7 @@
       </c>
       <c r="N37" s="25" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="O37" s="21" t="inlineStr">
@@ -3916,7 +3912,7 @@
       </c>
       <c r="N38" s="13" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="O38" s="21" t="inlineStr">
@@ -4008,7 +4004,7 @@
       </c>
       <c r="N39" s="25" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.38s</t>
         </is>
       </c>
       <c r="O39" s="21" t="inlineStr">
@@ -4273,7 +4269,7 @@
       <c r="M42" s="34" t="n"/>
       <c r="N42" s="13" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="O42" s="21" t="inlineStr">
@@ -4345,7 +4341,7 @@
       <c r="M43" s="35" t="n"/>
       <c r="N43" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O43" s="21" t="inlineStr">
@@ -4654,7 +4650,7 @@
       </c>
       <c r="N47" s="25" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O47" s="21" t="inlineStr">
@@ -4902,7 +4898,7 @@
       </c>
       <c r="N50" s="13" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.14s</t>
         </is>
       </c>
       <c r="O50" s="21" t="inlineStr">
@@ -5001,7 +4997,7 @@
       </c>
       <c r="N51" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O51" s="21" t="inlineStr">
@@ -5588,7 +5584,7 @@
       <c r="M58" s="34" t="n"/>
       <c r="N58" s="13" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O58" s="21" t="inlineStr">
@@ -5789,7 +5785,7 @@
       </c>
       <c r="N60" s="13" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O60" s="21" t="inlineStr">
@@ -5873,7 +5869,7 @@
       </c>
       <c r="N61" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O61" s="21" t="inlineStr">
@@ -6142,7 +6138,7 @@
       </c>
       <c r="N64" s="13" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.03s</t>
         </is>
       </c>
       <c r="O64" s="21" t="inlineStr">
@@ -6233,7 +6229,7 @@
       <c r="M65" s="35" t="n"/>
       <c r="N65" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O65" s="21" t="inlineStr">
@@ -6311,7 +6307,7 @@
       <c r="M66" s="34" t="n"/>
       <c r="N66" s="13" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O66" s="21" t="inlineStr">
@@ -6393,7 +6389,7 @@
       </c>
       <c r="N67" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O67" s="21" t="inlineStr">
@@ -6649,7 +6645,7 @@
       <c r="M70" s="34" t="n"/>
       <c r="N70" s="13" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O70" s="21" t="inlineStr">
@@ -6727,7 +6723,7 @@
       </c>
       <c r="N71" s="25" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O71" s="21" t="inlineStr">
@@ -6805,7 +6801,7 @@
       </c>
       <c r="N72" s="13" t="inlineStr">
         <is>
-          <t>0.07s</t>
+          <t>0.08s</t>
         </is>
       </c>
       <c r="O72" s="21" t="inlineStr">
@@ -7288,7 +7284,7 @@
       </c>
       <c r="N78" s="13" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O78" s="21" t="inlineStr">
@@ -8214,7 +8210,7 @@
       </c>
       <c r="N89" s="25" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O89" s="21" t="inlineStr">
@@ -10998,7 +10994,7 @@
       </c>
       <c r="N125" s="39" t="inlineStr">
         <is>
-          <t>0.03s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O125" s="41" t="inlineStr">
@@ -11166,7 +11162,7 @@
       </c>
       <c r="N127" s="39" t="inlineStr">
         <is>
-          <t>0.03s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O127" s="41" t="inlineStr">
@@ -11892,7 +11888,7 @@
       </c>
       <c r="N136" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O136" s="41" t="inlineStr">
@@ -12208,7 +12204,7 @@
       </c>
       <c r="N140" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O140" s="41" t="inlineStr">
@@ -12682,7 +12678,7 @@
       </c>
       <c r="N146" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O146" s="41" t="inlineStr">
@@ -12761,7 +12757,7 @@
       </c>
       <c r="N147" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O147" s="41" t="inlineStr">
@@ -12840,7 +12836,7 @@
       </c>
       <c r="N148" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O148" s="41" t="inlineStr">
@@ -12919,7 +12915,7 @@
       </c>
       <c r="N149" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O149" s="41" t="inlineStr">
@@ -13234,7 +13230,7 @@
       </c>
       <c r="N153" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O153" s="41" t="inlineStr">
@@ -13471,7 +13467,7 @@
       </c>
       <c r="N156" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O156" s="41" t="inlineStr">
@@ -13548,7 +13544,7 @@
       </c>
       <c r="N157" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O157" s="41" t="inlineStr">
@@ -13702,7 +13698,7 @@
       </c>
       <c r="N159" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O159" s="41" t="inlineStr">
@@ -13856,7 +13852,7 @@
       </c>
       <c r="N161" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O161" s="41" t="inlineStr">
@@ -14010,7 +14006,7 @@
       </c>
       <c r="N163" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O163" s="41" t="inlineStr">
@@ -14165,7 +14161,7 @@
       </c>
       <c r="N165" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O165" s="41" t="inlineStr">
@@ -15089,7 +15085,7 @@
       </c>
       <c r="N176" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O176" s="41" t="inlineStr">
@@ -15493,7 +15489,7 @@
       </c>
       <c r="N181" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O181" s="41" t="inlineStr">
@@ -16696,7 +16692,7 @@
       </c>
       <c r="N196" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O196" s="41" t="inlineStr">
@@ -16773,7 +16769,7 @@
       </c>
       <c r="N197" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O197" s="41" t="inlineStr">
@@ -17543,7 +17539,7 @@
       </c>
       <c r="N207" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O207" s="41" t="inlineStr">
@@ -18129,7 +18125,7 @@
       </c>
       <c r="N214" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O214" s="41" t="inlineStr">
@@ -19243,7 +19239,7 @@
       </c>
       <c r="N228" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O228" s="41" t="inlineStr">
@@ -19322,7 +19318,7 @@
       </c>
       <c r="N229" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O229" s="41" t="inlineStr">
@@ -19401,7 +19397,7 @@
       </c>
       <c r="N230" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O230" s="41" t="inlineStr">
@@ -20124,7 +20120,7 @@
       </c>
       <c r="N239" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O239" s="41" t="inlineStr">
@@ -20201,7 +20197,7 @@
       </c>
       <c r="N240" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O240" s="41" t="inlineStr">
@@ -20278,7 +20274,7 @@
       </c>
       <c r="N241" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O241" s="41" t="inlineStr">
@@ -20355,7 +20351,7 @@
       </c>
       <c r="N242" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O242" s="41" t="inlineStr">
@@ -20894,7 +20890,7 @@
       </c>
       <c r="N249" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O249" s="41" t="inlineStr">
@@ -21055,7 +21051,7 @@
       </c>
       <c r="N251" s="39" t="inlineStr">
         <is>
-          <t>0.03s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O251" s="41" t="inlineStr">
@@ -21221,7 +21217,7 @@
       </c>
       <c r="N253" s="39" t="inlineStr">
         <is>
-          <t>0.03s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O253" s="41" t="inlineStr">
@@ -21397,7 +21393,7 @@
       </c>
       <c r="N255" s="39" t="inlineStr">
         <is>
-          <t>0.03s</t>
+          <t>0.04s</t>
         </is>
       </c>
       <c r="O255" s="41" t="inlineStr">
@@ -21562,7 +21558,7 @@
       </c>
       <c r="N257" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O257" s="41" t="inlineStr">
@@ -21719,7 +21715,7 @@
       </c>
       <c r="N259" s="39" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.12s</t>
         </is>
       </c>
       <c r="O259" s="41" t="inlineStr">
@@ -22273,7 +22269,7 @@
       </c>
       <c r="N266" s="39" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.04s</t>
         </is>
       </c>
       <c r="O266" s="41" t="inlineStr">
@@ -22349,7 +22345,7 @@
       </c>
       <c r="N267" s="39" t="inlineStr">
         <is>
-          <t>0.04s</t>
+          <t>0.05s</t>
         </is>
       </c>
       <c r="O267" s="41" t="inlineStr">
@@ -22746,7 +22742,7 @@
       </c>
       <c r="N272" s="39" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.04s</t>
         </is>
       </c>
       <c r="O272" s="41" t="inlineStr">
@@ -24694,7 +24690,7 @@
       </c>
       <c r="N297" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O297" s="41" t="inlineStr">
@@ -24928,7 +24924,7 @@
       </c>
       <c r="N300" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O300" s="41" t="inlineStr">
@@ -25636,7 +25632,7 @@
       </c>
       <c r="N309" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O309" s="41" t="inlineStr">
@@ -26259,7 +26255,7 @@
       </c>
       <c r="N317" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O317" s="41" t="inlineStr">
@@ -26337,7 +26333,7 @@
       </c>
       <c r="N318" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O318" s="41" t="inlineStr">
@@ -26415,7 +26411,7 @@
       </c>
       <c r="N319" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O319" s="41" t="inlineStr">
@@ -26573,7 +26569,7 @@
       </c>
       <c r="N321" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O321" s="41" t="inlineStr">
@@ -27142,7 +27138,7 @@
       </c>
       <c r="N328" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O328" s="41" t="inlineStr">
@@ -27766,7 +27762,7 @@
       </c>
       <c r="N336" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O336" s="41" t="inlineStr">
@@ -27845,7 +27841,7 @@
       </c>
       <c r="N337" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O337" s="41" t="inlineStr">
@@ -29702,7 +29698,7 @@
       <c r="G361" s="39" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาชั้นปีสุดท้ายที่เหลือรายวิชาไม่ถึง 9 หน่วยกิต หรือต้องลงเกิน 22 หน่วยกิตเพื่อสำเร็จการศึกษา สามารถลงทะเบียนได้สูงสุดไม่เกิน 27 หน่วยกิต โดยต้องได้รับอนุมัติจากสภาวิชาการ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 ซึ่งระบุไว้ชัดเจนว่า ข้อยกเว้นสำหรับนักศึกษาชั้นปีสุดท้ายสามารถลงทะเบียนได้สูงสุด 27 หน่วยกิต</t>
+นักศึกษาชั้นปีสุดท้ายที่เหลือรายวิชาไม่ถึง 9 หน่วยกิต หรือต้องลงเกิน 22 หน่วยกิตเพื่อสำเร็จการศึกษา สามารถลงทะเบียนได้สูงสุดไม่เกิน 27 หน่วยกิต โดยต้องได้รับอนุมัติจากสภาวิชาการ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 ซึ่งระบุไว้ชัดเจนสำหรับกรณีปีสุดท้าย</t>
         </is>
       </c>
       <c r="H361" s="39" t="inlineStr">
@@ -29735,7 +29731,7 @@
       </c>
       <c r="N361" s="39" t="inlineStr">
         <is>
-          <t>2.20s</t>
+          <t>1.51s</t>
         </is>
       </c>
       <c r="O361" s="41" t="inlineStr">
@@ -30688,7 +30684,7 @@
       </c>
       <c r="N373" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O373" s="41" t="inlineStr">
@@ -30843,7 +30839,7 @@
       </c>
       <c r="N375" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O375" s="41" t="inlineStr">
@@ -32008,7 +32004,7 @@
       </c>
       <c r="N390" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O390" s="41" t="inlineStr">
@@ -32087,7 +32083,7 @@
       </c>
       <c r="N391" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O391" s="41" t="inlineStr">
@@ -32558,7 +32554,7 @@
       </c>
       <c r="N397" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O397" s="41" t="inlineStr">
@@ -33196,7 +33192,7 @@
       </c>
       <c r="N405" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O405" s="41" t="inlineStr">
@@ -33350,7 +33346,7 @@
       </c>
       <c r="N407" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O407" s="41" t="inlineStr">
@@ -33504,7 +33500,7 @@
       </c>
       <c r="N409" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O409" s="41" t="inlineStr">
@@ -36267,7 +36263,7 @@
       </c>
       <c r="N444" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O444" s="41" t="inlineStr">
@@ -36346,7 +36342,7 @@
       </c>
       <c r="N445" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O445" s="41" t="inlineStr">
@@ -36423,7 +36419,7 @@
       </c>
       <c r="N446" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O446" s="41" t="inlineStr">
@@ -36577,7 +36573,7 @@
       </c>
       <c r="N448" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O448" s="41" t="inlineStr">
@@ -36820,7 +36816,7 @@
       </c>
       <c r="N451" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O451" s="41" t="inlineStr">
@@ -37445,7 +37441,7 @@
       </c>
       <c r="N459" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O459" s="41" t="inlineStr">
@@ -39175,7 +39171,7 @@
       </c>
       <c r="N481" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O481" s="41" t="inlineStr">
@@ -39881,7 +39877,7 @@
       </c>
       <c r="N490" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O490" s="41" t="inlineStr">
@@ -40195,7 +40191,7 @@
       </c>
       <c r="N494" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O494" s="41" t="inlineStr">
@@ -40349,7 +40345,7 @@
       </c>
       <c r="N496" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O496" s="41" t="inlineStr">
@@ -40675,7 +40671,7 @@
       </c>
       <c r="N500" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O500" s="41" t="inlineStr">
@@ -40912,7 +40908,7 @@
       </c>
       <c r="N503" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O503" s="41" t="inlineStr">
@@ -40991,7 +40987,7 @@
       </c>
       <c r="N504" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O504" s="41" t="inlineStr">
@@ -41147,7 +41143,7 @@
       </c>
       <c r="N506" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O506" s="41" t="inlineStr">
@@ -41224,7 +41220,7 @@
       </c>
       <c r="N507" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O507" s="41" t="inlineStr">
@@ -41390,7 +41386,7 @@
       </c>
       <c r="N509" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O509" s="41" t="inlineStr">
@@ -41469,7 +41465,7 @@
       </c>
       <c r="N510" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O510" s="41" t="inlineStr">
@@ -41627,7 +41623,7 @@
       </c>
       <c r="N512" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O512" s="41" t="inlineStr">
@@ -42441,7 +42437,7 @@
       </c>
       <c r="N522" s="39" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.53s</t>
         </is>
       </c>
       <c r="O522" s="41" t="inlineStr">
@@ -42519,7 +42515,7 @@
       </c>
       <c r="N523" s="39" t="inlineStr">
         <is>
-          <t>0.04s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O523" s="41" t="inlineStr">
@@ -42683,7 +42679,7 @@
       </c>
       <c r="N525" s="39" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="O525" s="41" t="inlineStr">
@@ -43002,7 +42998,7 @@
       </c>
       <c r="N529" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O529" s="41" t="inlineStr">
@@ -43474,7 +43470,7 @@
       </c>
       <c r="N535" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O535" s="41" t="inlineStr">
@@ -44334,7 +44330,7 @@
       </c>
       <c r="N546" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O546" s="41" t="inlineStr">
@@ -44413,7 +44409,7 @@
       </c>
       <c r="N547" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O547" s="41" t="inlineStr">
@@ -44570,7 +44566,7 @@
       </c>
       <c r="N549" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O549" s="41" t="inlineStr">
@@ -44930,7 +44926,7 @@
       </c>
       <c r="N553" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O553" s="41" t="inlineStr">
@@ -45262,7 +45258,7 @@
       </c>
       <c r="N557" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O557" s="41" t="inlineStr">
@@ -45346,7 +45342,7 @@
       </c>
       <c r="N558" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O558" s="41" t="inlineStr">
@@ -46059,7 +46055,7 @@
       </c>
       <c r="N567" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O567" s="41" t="inlineStr">
@@ -46138,7 +46134,7 @@
       </c>
       <c r="N568" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O568" s="41" t="inlineStr">
@@ -46246,7 +46242,7 @@
       </c>
       <c r="N569" s="39" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="O569" s="41" t="inlineStr">
@@ -47115,7 +47111,7 @@
       </c>
       <c r="N580" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O580" s="41" t="inlineStr">
@@ -48611,7 +48607,7 @@
       </c>
       <c r="N599" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O599" s="41" t="inlineStr">
@@ -48654,7 +48650,7 @@
       <c r="G600" s="39" t="inlineStr">
         <is>
           <t>ไม่ได้  
-นักศึกษาทั่วไปต้องลงทะเบียนไม่เกิน 22 หน่วยกิตต่อภาคการศึกษาปกติ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (หน้า 82) แม้จะเป็นนักศึกษาชั้นปีสุดท้ายก็ยังจำกัดที่ 27 หน่วยกิต แต่ต้องมีเหตุผลเฉพาะเจาะจง และต้องได้รับอนุมัติจากสภาวิชาการ ซึ่งไม่ได้ระบุว่าสามารถลง 25 หน่วยกิตได้โดยอัตโนมัติ</t>
+นักศึกษาทั่วไปต้องลงทะเบียนไม่เกิน 22 หน่วยกิตต่อภาคการศึกษาปกติ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 แม้จะเป็นนักศึกษาชั้นปีสุดท้ายก็ตาม แต่ต้องไม่เกิน 27 หน่วยกิต หากมีข้อยกเว้นเฉพาะกรณีที่เหลือรายวิชาไม่ถึง 3 หน่วยกิต หรือต้องลงเพื่อสำเร็จการศึกษา ซึ่งไม่ได้ระบุว่าเป็นกรณีนี้ ดังนั้นการลง 25 หน่วยกิตเกินข้อจำกัดปกติ และไม่มีหลักฐานยืนยันว่าเข้าข่ายข้อยกเว้น</t>
         </is>
       </c>
       <c r="H600" s="39" t="inlineStr">
@@ -48687,7 +48683,7 @@
       </c>
       <c r="N600" s="39" t="inlineStr">
         <is>
-          <t>1.47s</t>
+          <t>2.24s</t>
         </is>
       </c>
       <c r="O600" s="41" t="inlineStr">
@@ -48767,7 +48763,7 @@
       </c>
       <c r="N601" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O601" s="41" t="inlineStr">
@@ -48921,7 +48917,7 @@
       </c>
       <c r="N603" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O603" s="41" t="inlineStr">
@@ -48998,7 +48994,7 @@
       </c>
       <c r="N604" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O604" s="41" t="inlineStr">
@@ -49157,7 +49153,7 @@
       </c>
       <c r="N606" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O606" s="41" t="inlineStr">
@@ -49235,7 +49231,7 @@
       </c>
       <c r="N607" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O607" s="41" t="inlineStr">
@@ -49312,7 +49308,7 @@
       </c>
       <c r="N608" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O608" s="41" t="inlineStr">
@@ -49469,7 +49465,7 @@
       </c>
       <c r="N610" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O610" s="41" t="inlineStr">
@@ -49546,7 +49542,7 @@
       </c>
       <c r="N611" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O611" s="41" t="inlineStr">
@@ -51007,7 +51003,7 @@
       <c r="G630" s="39" t="inlineStr">
         <is>
           <t>ไม่ได้  
-นักศึกษาต้องลงทะเบียนไม่น้อยกว่า 9 หน่วยกิตในภาคการศึกษาปกติ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 ซึ่งเป็นข้อกำหนดบังคับสำหรับทุกหลักสูตรปริญญาตรี ไม่ใช่ข้อยกเว้นเฉพาะหลักสูตร DSBA</t>
+นักศึกษาต้องลงทะเบียนไม่น้อยกว่า 9 หน่วยกิตในภาคการศึกษาปกติ ตามข้อบังคับสถาบันเทคโนโลยีพระจอมเกล้าเจ้าคุณทหารลาดกระบัง ว่าด้วยการศึกษาระดับปริญญาตรี พ.ศ. 2564 (ภาคผนวก ก) ซึ่งใช้กับหลักสูตรวท.บ. (วิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ) คณะเทคโนโลยีสารสนเทศ สจล. ทุกภาคการศึกษาปกติ</t>
         </is>
       </c>
       <c r="H630" s="39" t="inlineStr">
@@ -51040,7 +51036,7 @@
       </c>
       <c r="N630" s="39" t="inlineStr">
         <is>
-          <t>1.41s</t>
+          <t>1.61s</t>
         </is>
       </c>
       <c r="O630" s="41" t="inlineStr">
@@ -51083,7 +51079,9 @@
       <c r="G631" s="39" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาสามารถลงทะเบียนเรียนได้ไม่เกิน 9 หน่วยกิตในภาคการศึกษาพิเศษ (ซัมเมอร์) ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 หากลงฝึกงานในภาคพิเศษ จะไม่สามารถลงวิชาอื่นได้ในภาคเดียวกัน เนื่องจากเป็นข้อห้ามโดยตรงในข้อบังคับดังกล่าว</t>
+นักศึกษาสามารถลงทะเบียนเรียนได้ไม่เกิน 9 หน่วยกิตในภาคการศึกษาพิเศษ (ภาคฤดูร้อน) ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82  
+หากลงฝึกงานในภาคพิเศษ ห้ามลงทะเบียนเรียนรายวิชาอื่นเพิ่มเติมได้  
+ประเภทวิชา: ภาคการศึกษาพิเศษ, ข้อบังคับการลงทะเบียนเรียน</t>
         </is>
       </c>
       <c r="H631" s="39" t="inlineStr">
@@ -51116,7 +51114,7 @@
       </c>
       <c r="N631" s="39" t="inlineStr">
         <is>
-          <t>1.52s</t>
+          <t>1.75s</t>
         </is>
       </c>
       <c r="O631" s="41" t="inlineStr">
@@ -51356,34 +51354,2182 @@
         </is>
       </c>
     </row>
-    <row r="635" ht="14.25" customHeight="1" s="36"/>
-    <row r="636" ht="14.25" customHeight="1" s="36"/>
-    <row r="637" ht="14.25" customHeight="1" s="36"/>
-    <row r="638" ht="14.25" customHeight="1" s="36"/>
-    <row r="639" ht="14.25" customHeight="1" s="36"/>
-    <row r="640" ht="14.25" customHeight="1" s="36"/>
-    <row r="641" ht="14.25" customHeight="1" s="36"/>
-    <row r="642" ht="14.25" customHeight="1" s="36"/>
-    <row r="643" ht="14.25" customHeight="1" s="36"/>
-    <row r="644" ht="14.25" customHeight="1" s="36"/>
-    <row r="645" ht="14.25" customHeight="1" s="36"/>
-    <row r="646" ht="14.25" customHeight="1" s="36"/>
-    <row r="647" ht="14.25" customHeight="1" s="36"/>
-    <row r="648" ht="14.25" customHeight="1" s="36"/>
-    <row r="649" ht="14.25" customHeight="1" s="36"/>
-    <row r="650" ht="14.25" customHeight="1" s="36"/>
-    <row r="651" ht="14.25" customHeight="1" s="36"/>
-    <row r="652" ht="14.25" customHeight="1" s="36"/>
-    <row r="653" ht="14.25" customHeight="1" s="36"/>
-    <row r="654" ht="14.25" customHeight="1" s="36"/>
-    <row r="655" ht="14.25" customHeight="1" s="36"/>
-    <row r="656" ht="14.25" customHeight="1" s="36"/>
-    <row r="657" ht="14.25" customHeight="1" s="36"/>
-    <row r="658" ht="14.25" customHeight="1" s="36"/>
-    <row r="659" ht="14.25" customHeight="1" s="36"/>
-    <row r="660" ht="14.25" customHeight="1" s="36"/>
-    <row r="661" ht="14.25" customHeight="1" s="36"/>
-    <row r="662" ht="14.25" customHeight="1" s="36"/>
+    <row r="635" ht="14.25" customHeight="1" s="36">
+      <c r="A635" s="37" t="inlineStr">
+        <is>
+          <t>QH1</t>
+        </is>
+      </c>
+      <c r="B635" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C635" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D635" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าลงตามแผน ปี 3 เทอม 1 ทั้งเทอมรวมกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E635" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F635" s="39" t="inlineStr">
+        <is>
+          <t>18 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G635" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 3 ภาคการศึกษาที่ 1 ตามแผนปกติของ AIT 2566 (ปริญญาตรี) ลงรวม 18 หน่วยกิต
+- จากบรรทัด 'รวม' ของภาคนี้ในตารางแผนการศึกษา หน้า 25 (รวมวิชาเลือก/ศึกษาทั่วไปที่แผนกำหนดไว้แล้ว ไม่ใช่เฉพาะวิชาบังคับ)</t>
+        </is>
+      </c>
+      <c r="H635" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 25</t>
+        </is>
+      </c>
+      <c r="I635" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของภาคตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J635" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K635" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L635" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M635" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N635" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O635" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="636" ht="14.25" customHeight="1" s="36">
+      <c r="A636" s="37" t="inlineStr">
+        <is>
+          <t>QH2</t>
+        </is>
+      </c>
+      <c r="B636" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C636" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D636" s="39" t="inlineStr">
+        <is>
+          <t>วิชาที่ต้องผ่านก่อนลงการเรียนรู้ของเครื่องเชิงความน่าจะเป็น คือวิชาอะไร แล้ววิชานั้นอยู่ปีไหนเทอมไหน</t>
+        </is>
+      </c>
+      <c r="E636" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F636" s="39" t="inlineStr">
+        <is>
+          <t>06066001 ปี 1 ภาค 1</t>
+        </is>
+      </c>
+      <c r="G636" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06066001 ความน่าจะเป็นและสถิติ (PROBABILITY AND STATISTICS) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H636" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 37, 291, 19, 20, 23, 24, 289</t>
+        </is>
+      </c>
+      <c r="I636" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J636" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="K636" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L636" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M636" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N636" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O636" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="637" ht="14.25" customHeight="1" s="36">
+      <c r="A637" s="37" t="inlineStr">
+        <is>
+          <t>QH3</t>
+        </is>
+      </c>
+      <c r="B637" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C637" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D637" s="39" t="inlineStr">
+        <is>
+          <t>ก่อนจะลงวิชาการเรียนรู้ของเครื่องเชิงความน่าจะเป็น ต้องสอบผ่านวิชาอะไรมาก่อน และตัววิชานี้อยู่ในแผนปีไหน</t>
+        </is>
+      </c>
+      <c r="E637" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F637" s="39" t="inlineStr">
+        <is>
+          <t>06066001; ปี 2 ภาค 1</t>
+        </is>
+      </c>
+      <c r="G637" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06066001 ความน่าจะเป็นและสถิติ (PROBABILITY AND STATISTICS) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H637" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 37, 291, 19, 20, 23, 24, 289</t>
+        </is>
+      </c>
+      <c r="I637" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J637" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="K637" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L637" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M637" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N637" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O637" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="638" ht="14.25" customHeight="1" s="36">
+      <c r="A638" s="37" t="inlineStr">
+        <is>
+          <t>QC1</t>
+        </is>
+      </c>
+      <c r="B638" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C638" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D638" s="39" t="inlineStr">
+        <is>
+          <t>เทอมเดียวกันจะลงแคลคูลัส 2 พร้อมกับพื้นฐานการเรียนรู้เชิงลึก เลยได้ไหม</t>
+        </is>
+      </c>
+      <c r="E638" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F638" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ได้ ต้องผ่าน 06046401 ก่อน</t>
+        </is>
+      </c>
+      <c r="G638" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ไม่ได้ — ต้องสอบผ่าน 06046401 แคลคูลัส 2 ก่อน จึงจะลง 06046406 พื้นฐานการเรียนรู้เชิงลึก ได้ จึงลงพร้อมกันในภาคเดียวกันไม่ได้
+- 06046401 แคลคูลัส 2 (CALCULUS 2) — ปีที่ 1 ภาคการศึกษาที่ 2
+- 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING) — ปีที่ 2 ภาคการศึกษาที่ 1
+- 06046406 มีวิชาบังคับก่อนเป็น 06046401 (ต้องสอบผ่าน 06046401 ก่อนจึงลง 06046406 ได้)</t>
+        </is>
+      </c>
+      <c r="H638" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 37, 292, 19, 20, 23, 24, 287</t>
+        </is>
+      </c>
+      <c r="I638" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบปี/ภาคของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J638" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="K638" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L638" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M638" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N638" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O638" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="639" ht="14.25" customHeight="1" s="36">
+      <c r="A639" s="37" t="inlineStr">
+        <is>
+          <t>QC2</t>
+        </is>
+      </c>
+      <c r="B639" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C639" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D639" s="39" t="inlineStr">
+        <is>
+          <t>ปี 2 ภาค 2 ตามแผนต้องลงกี่หน่วยกิต เกินเพดานที่ลงได้ต่อภาคปกติไหม</t>
+        </is>
+      </c>
+      <c r="E639" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F639" s="39" t="inlineStr">
+        <is>
+          <t>19 หน่วยกิต ไม่เกิน 22</t>
+        </is>
+      </c>
+      <c r="G639" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 2 ภาคการศึกษาที่ 2 ตามแผนปกติของ AIT 2566 (ปริญญาตรี) ลงรวม 19 หน่วยกิต
+- จากบรรทัด 'รวม' ของภาคนี้ในตารางแผนการศึกษา หน้า 24 (รวมวิชาเลือก/ศึกษาทั่วไปที่แผนกำหนดไว้แล้ว ไม่ใช่เฉพาะวิชาบังคับ)
+- ข้อบังคับ: ภาคการศึกษาปกติลงทะเบียนได้ 9–22 หน่วยกิต → 19 หน่วยกิต อยู่ในเกณฑ์ ไม่เกินเพดาน 22</t>
+        </is>
+      </c>
+      <c r="H639" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 24, 82</t>
+        </is>
+      </c>
+      <c r="I639" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของภาคตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J639" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K639" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L639" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M639" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N639" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O639" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="640" ht="14.25" customHeight="1" s="36">
+      <c r="A640" s="37" t="inlineStr">
+        <is>
+          <t>QH4</t>
+        </is>
+      </c>
+      <c r="B640" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C640" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D640" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าลงตามแผน ปี 3 เทอม 2 ทั้งเทอมรวมกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E640" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F640" s="39" t="inlineStr">
+        <is>
+          <t>9 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G640" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 3 ภาคการศึกษาที่ 2 ตามแผนปกติของ BIT 2565 (ปริญญาตรี) ลงรวม 12 หน่วยกิต
+- จากบรรทัด 'รวม' ของภาคนี้ในตารางแผนการศึกษา หน้า 29 (รวมวิชาเลือก/ศึกษาทั่วไปที่แผนกำหนดไว้แล้ว ไม่ใช่เฉพาะวิชาบังคับ)</t>
+        </is>
+      </c>
+      <c r="H640" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 29</t>
+        </is>
+      </c>
+      <c r="I640" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของภาคตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J640" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K640" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L640" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M640" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N640" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O640" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="641" ht="14.25" customHeight="1" s="36">
+      <c r="A641" s="37" t="inlineStr">
+        <is>
+          <t>QH5</t>
+        </is>
+      </c>
+      <c r="B641" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C641" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D641" s="39" t="inlineStr">
+        <is>
+          <t>วิชาที่ต้องผ่านก่อนลงการพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก คือวิชาอะไร แล้ววิชานั้นอยู่ปีไหนเทอมไหน</t>
+        </is>
+      </c>
+      <c r="E641" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F641" s="39" t="inlineStr">
+        <is>
+          <t>06036119 ปี 1 ภาค 2</t>
+        </is>
+      </c>
+      <c r="G641" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06036114 การพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก (WEB APPLICATION DEVELOPMENT USING FRAMEWORKS) — 3(2-2-5) | ปีที่ 3 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06036119 พื้นฐานการเขียนโปรแกรม (PROGRAMMING FUNDAMENTALS) — 3(2-2-5) | ปีที่ 1 ภาคการศึกษาที่ 2
+    • 06036122 การสื่อสารด้วยภาพสำหรับธุรกิจ (VISUAL COMMUNICATION FOR BUSINESS) — 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H641" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 75, 23, 244, 270, 22, 27, 28, 32</t>
+        </is>
+      </c>
+      <c r="I641" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J641" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K641" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L641" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M641" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N641" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O641" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="642" ht="14.25" customHeight="1" s="36">
+      <c r="A642" s="37" t="inlineStr">
+        <is>
+          <t>QH6</t>
+        </is>
+      </c>
+      <c r="B642" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C642" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D642" s="39" t="inlineStr">
+        <is>
+          <t>ก่อนจะลงวิชาการพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก ต้องสอบผ่านวิชาอะไรมาก่อน และตัววิชานี้อยู่ในแผนปีไหน</t>
+        </is>
+      </c>
+      <c r="E642" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F642" s="39" t="inlineStr">
+        <is>
+          <t>06036119, 06036122; ปี 3 ภาค 1</t>
+        </is>
+      </c>
+      <c r="G642" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06036114 การพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก (WEB APPLICATION DEVELOPMENT USING FRAMEWORKS) — 3(2-2-5) | ปีที่ 3 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06036119 พื้นฐานการเขียนโปรแกรม (PROGRAMMING FUNDAMENTALS) — 3(2-2-5) | ปีที่ 1 ภาคการศึกษาที่ 2
+    • 06036122 การสื่อสารด้วยภาพสำหรับธุรกิจ (VISUAL COMMUNICATION FOR BUSINESS) — 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H642" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 75, 23, 244, 270, 22, 27, 28, 32</t>
+        </is>
+      </c>
+      <c r="I642" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J642" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K642" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L642" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M642" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N642" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O642" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="643" ht="14.25" customHeight="1" s="36">
+      <c r="A643" s="37" t="inlineStr">
+        <is>
+          <t>QC3</t>
+        </is>
+      </c>
+      <c r="B643" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C643" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D643" s="39" t="inlineStr">
+        <is>
+          <t>เทอมเดียวกันจะลงการสื่อสารด้วยภาพสำหรับธุรกิจ พร้อมกับการพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก เลยได้ไหม</t>
+        </is>
+      </c>
+      <c r="E643" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F643" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ได้ ต้องผ่าน 06036122 ก่อน</t>
+        </is>
+      </c>
+      <c r="G643" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ไม่ได้ — ต้องสอบผ่าน 06036122 การสื่อสารด้วยภาพสำหรับธุรกิจ ก่อน จึงจะลง 06036114 การพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก ได้ จึงลงพร้อมกันในภาคเดียวกันไม่ได้
+- 06036122 การสื่อสารด้วยภาพสำหรับธุรกิจ (VISUAL COMMUNICATION FOR BUSINESS) — ปีที่ 2 ภาคการศึกษาที่ 1
+- 06036114 การพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก (WEB APPLICATION DEVELOPMENT USING FRAMEWORKS) — ปีที่ 3 ภาคการศึกษาที่ 1
+- 06036114 มีวิชาบังคับก่อนเป็น 06036122 (ต้องสอบผ่าน 06036122 ก่อนจึงลง 06036114 ได้)</t>
+        </is>
+      </c>
+      <c r="H643" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 75, 22, 23, 27, 28, 244, 247, 269</t>
+        </is>
+      </c>
+      <c r="I643" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบปี/ภาคของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J643" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K643" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L643" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M643" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N643" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O643" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="644" ht="14.25" customHeight="1" s="36">
+      <c r="A644" s="37" t="inlineStr">
+        <is>
+          <t>QC4</t>
+        </is>
+      </c>
+      <c r="B644" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C644" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D644" s="39" t="inlineStr">
+        <is>
+          <t>ปี 3 ภาค 1 ตามแผนต้องลงกี่หน่วยกิต เกินเพดานที่ลงได้ต่อภาคปกติไหม</t>
+        </is>
+      </c>
+      <c r="E644" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F644" s="39" t="inlineStr">
+        <is>
+          <t>18 หน่วยกิต ไม่เกิน 22</t>
+        </is>
+      </c>
+      <c r="G644" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 3 ภาคการศึกษาที่ 1 ตามแผนปกติของ BIT 2565 (ปริญญาตรี) ลงรวม 18 หน่วยกิต
+- จากบรรทัด 'รวม' ของภาคนี้ในตารางแผนการศึกษา หน้า 28 (รวมวิชาเลือก/ศึกษาทั่วไปที่แผนกำหนดไว้แล้ว ไม่ใช่เฉพาะวิชาบังคับ)
+- ข้อบังคับ: ภาคการศึกษาปกติลงทะเบียนได้ 9–22 หน่วยกิต → 18 หน่วยกิต อยู่ในเกณฑ์ ไม่เกินเพดาน 22</t>
+        </is>
+      </c>
+      <c r="H644" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 28, 82</t>
+        </is>
+      </c>
+      <c r="I644" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของภาคตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J644" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K644" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L644" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M644" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N644" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O644" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="645" ht="14.25" customHeight="1" s="36">
+      <c r="A645" s="37" t="inlineStr">
+        <is>
+          <t>QH7</t>
+        </is>
+      </c>
+      <c r="B645" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C645" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D645" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าลงตามแผน ปี 2 เทอม 2 ทั้งเทอมรวมกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E645" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F645" s="39" t="inlineStr">
+        <is>
+          <t>21 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G645" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 2 ภาคการศึกษาที่ 2 ตามแผนปกติของ DSBA 2565 (ปริญญาตรี) ลงรวม 21 หน่วยกิต
+- จากบรรทัด 'รวม' ของภาคนี้ในตารางแผนการศึกษา หน้า 26 (รวมวิชาเลือก/ศึกษาทั่วไปที่แผนกำหนดไว้แล้ว ไม่ใช่เฉพาะวิชาบังคับ)</t>
+        </is>
+      </c>
+      <c r="H645" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 26</t>
+        </is>
+      </c>
+      <c r="I645" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของภาคตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J645" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K645" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L645" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M645" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N645" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O645" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="646" ht="14.25" customHeight="1" s="36">
+      <c r="A646" s="37" t="inlineStr">
+        <is>
+          <t>QH8</t>
+        </is>
+      </c>
+      <c r="B646" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C646" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D646" s="39" t="inlineStr">
+        <is>
+          <t>วิชาที่ต้องผ่านก่อนลงแคลคูลัส 2 คือวิชาอะไร แล้ววิชานั้นอยู่ปีไหนเทอมไหน</t>
+        </is>
+      </c>
+      <c r="E646" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F646" s="39" t="inlineStr">
+        <is>
+          <t>06026200 ปี 1 ภาค 1</t>
+        </is>
+      </c>
+      <c r="G646" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06026201 แคลคูลัส 2 (CALCULUS 2) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06026200 แคลคูลัส 1 (CALCULUS 1) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H646" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 17, 68, 314, 353, 23, 24, 30, 31</t>
+        </is>
+      </c>
+      <c r="I646" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J646" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K646" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L646" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M646" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N646" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O646" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="647" ht="14.25" customHeight="1" s="36">
+      <c r="A647" s="37" t="inlineStr">
+        <is>
+          <t>QH9</t>
+        </is>
+      </c>
+      <c r="B647" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C647" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D647" s="39" t="inlineStr">
+        <is>
+          <t>ก่อนจะลงวิชาโครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 ต้องสอบผ่านวิชาอะไรมาก่อน และตัววิชานี้อยู่ในแผนปีไหน</t>
+        </is>
+      </c>
+      <c r="E647" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F647" s="39" t="inlineStr">
+        <is>
+          <t>06026214; ปี 4 ภาค 1</t>
+        </is>
+      </c>
+      <c r="G647" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06026215 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 2 (PROJECT IN DATA SCIENCE AND BUSINESS ANALYTICS 2) — 3(0-9-0) | ปีที่ 4 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06026214 โครงงานวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ 1 (PROJECT IN DATA SCIENCE AND BUSINESS ANALYTICS 1) — 3(0-9-0) | ปีที่ 3 ภาคการศึกษาที่ 2</t>
+        </is>
+      </c>
+      <c r="H647" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 19, 69, 325, 354, 28, 29, 35, 36</t>
+        </is>
+      </c>
+      <c r="I647" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J647" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K647" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L647" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M647" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N647" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O647" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="648" ht="14.25" customHeight="1" s="36">
+      <c r="A648" s="37" t="inlineStr">
+        <is>
+          <t>QC5</t>
+        </is>
+      </c>
+      <c r="B648" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C648" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D648" s="39" t="inlineStr">
+        <is>
+          <t>เทอมเดียวกันจะลงแนวคิดระบบฐานข้อมูล พร้อมกับระบบข้อมูลมหัต เลยได้ไหม</t>
+        </is>
+      </c>
+      <c r="E648" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F648" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ได้ ต้องผ่าน 06066300 ก่อน</t>
+        </is>
+      </c>
+      <c r="G648" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ไม่ได้ — ต้องสอบผ่าน 06066300 แนวคิดระบบฐานข้อมูล ก่อน จึงจะลง 06026213 ระบบข้อมูลมหัต ได้ จึงลงพร้อมกันในภาคเดียวกันไม่ได้
+- 06066300 แนวคิดระบบฐานข้อมูล (DATABASE SYSTEM CONCEPTS) — ปีที่ 2 ภาคการศึกษาที่ 1
+- 06026213 ระบบข้อมูลมหัต (BIG DATA SYSTEMS) — ปีที่ 3 ภาคการศึกษาที่ 2
+- 06026213 มีวิชาบังคับก่อนเป็น 06066300 (ต้องสอบผ่าน 06066300 ก่อนจึงลง 06026213 ได้)</t>
+        </is>
+      </c>
+      <c r="H648" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 18, 19, 25, 28, 32, 35, 69, 73</t>
+        </is>
+      </c>
+      <c r="I648" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบปี/ภาคของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J648" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K648" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L648" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M648" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N648" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O648" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="649" ht="14.25" customHeight="1" s="36">
+      <c r="A649" s="37" t="inlineStr">
+        <is>
+          <t>QH10</t>
+        </is>
+      </c>
+      <c r="B649" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C649" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D649" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าลงตามแผน ปี 2 เทอม 1 ทั้งเทอมรวมกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E649" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F649" s="39" t="inlineStr">
+        <is>
+          <t>18 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G649" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 2 ภาคการศึกษาที่ 1 ตามแผนปกติของ IT 2565 (ปริญญาตรี) ลงรวม 18 หน่วยกิต
+- จากบรรทัด 'รวม' ของภาคนี้ในตารางแผนการศึกษา หน้า 33 (รวมวิชาเลือก/ศึกษาทั่วไปที่แผนกำหนดไว้แล้ว ไม่ใช่เฉพาะวิชาบังคับ)</t>
+        </is>
+      </c>
+      <c r="H649" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 33</t>
+        </is>
+      </c>
+      <c r="I649" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของภาคตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J649" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K649" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L649" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M649" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N649" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O649" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="650" ht="14.25" customHeight="1" s="36">
+      <c r="A650" s="37" t="inlineStr">
+        <is>
+          <t>QH11</t>
+        </is>
+      </c>
+      <c r="B650" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C650" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D650" s="39" t="inlineStr">
+        <is>
+          <t>วิชาที่ต้องผ่านก่อนลงอินเทอร์เน็ตของสรรพสิ่ง คือวิชาอะไร แล้ววิชานั้นอยู่ปีไหนเทอมไหน</t>
+        </is>
+      </c>
+      <c r="E650" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F650" s="39" t="inlineStr">
+        <is>
+          <t>06016413 ปี 2 ภาค 1</t>
+        </is>
+      </c>
+      <c r="G650" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06016422 อินเทอร์เน็ตของสรรพสิ่ง (INTERNET OF THINGS) — 3(2-2-5) | ปีที่ 3 ภาคการศึกษาที่ 1
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06016413 ระบบเครือข่ายเบื้องต้น (INTRODUCTION TO NETWORK SYSTEMS) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H650" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 84, 333, 24, 25, 33, 35, 40, 328</t>
+        </is>
+      </c>
+      <c r="I650" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J650" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K650" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L650" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M650" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N650" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O650" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="651" ht="14.25" customHeight="1" s="36">
+      <c r="A651" s="37" t="inlineStr">
+        <is>
+          <t>QH12</t>
+        </is>
+      </c>
+      <c r="B651" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C651" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D651" s="39" t="inlineStr">
+        <is>
+          <t>ก่อนจะลงวิชาระบบโครงสร้างพื้นฐานและการบริการ ต้องสอบผ่านวิชาอะไรมาก่อน และตัววิชานี้อยู่ในแผนปีไหน</t>
+        </is>
+      </c>
+      <c r="E651" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F651" s="39" t="inlineStr">
+        <is>
+          <t>06016413; ปี 2 ภาค 2</t>
+        </is>
+      </c>
+      <c r="G651" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06016420 ระบบโครงสร้างพื้นฐานและการบริการ (INFRASTRUCTURE SYSTEMS AND SERVICES) — 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 2
+  ต้องผ่านวิชาบังคับก่อน:
+    • 06016413 ระบบเครือข่ายเบื้องต้น (INTRODUCTION TO NETWORK SYSTEMS) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H651" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 84, 24, 25, 33, 34, 40, 328, 331</t>
+        </is>
+      </c>
+      <c r="I651" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (prerequisite) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J651" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K651" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L651" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M651" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N651" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O651" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="652" ht="14.25" customHeight="1" s="36">
+      <c r="A652" s="37" t="inlineStr">
+        <is>
+          <t>QC6</t>
+        </is>
+      </c>
+      <c r="B652" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C652" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D652" s="39" t="inlineStr">
+        <is>
+          <t>เทอมเดียวกันจะลงการเขียนโปรแกรมเว็บพื้นฐาน พร้อมกับการออกแบบเว็บ เลยได้ไหม</t>
+        </is>
+      </c>
+      <c r="E652" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F652" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ได้ ต้องผ่าน 06066302 ก่อน</t>
+        </is>
+      </c>
+      <c r="G652" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ไม่ได้ — ต้องสอบผ่าน 06066302 การเขียนโปรแกรมเว็บพื้นฐาน ก่อน จึงจะลง 06016444 การออกแบบเว็บ ได้ จึงลงพร้อมกันในภาคเดียวกันไม่ได้
+- 06066302 การเขียนโปรแกรมเว็บพื้นฐาน (FUNDAMENTAL WEB PROGRAMMING) — ปีที่ 2 ภาคการศึกษาที่ 2
+- 06016444 การออกแบบเว็บ (WEB DESIGN) — ไม่ได้กำหนดปี/ภาคในแผนการศึกษา (วิชาเลือก)
+- 06016444 มีวิชาบังคับก่อนเป็น 06066302 (ต้องสอบผ่าน 06066302 ก่อนจึงลง 06016444 ได้)</t>
+        </is>
+      </c>
+      <c r="H652" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 342, 24, 27, 34, 41, 85, 88, 336</t>
+        </is>
+      </c>
+      <c r="I652" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบปี/ภาคของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J652" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K652" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L652" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M652" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N652" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O652" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="653" ht="14.25" customHeight="1" s="36">
+      <c r="A653" s="37" t="inlineStr">
+        <is>
+          <t>QH13</t>
+        </is>
+      </c>
+      <c r="B653" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C653" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D653" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเลือกแผนสหกิจศึกษา จะได้ออกไปสหกิจตอนปีไหน เทอมไหน และวิชาสหกิจกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E653" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F653" s="39" t="inlineStr">
+        <is>
+          <t>ปี 4 ภาค 2 6 หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="G653" s="39" t="inlineStr">
+        <is>
+          <t>รายวิชาที่มีเฉพาะในแผนที่เข้าโครงการสหกิจศึกษา (BIT 2565 (ปริญญาตรี)):
+- 06036147 สหกิจศึกษา — 6(0-35-0) | ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 35)
+- 06036148 สหกิจศึกษาต่างประเทศ — 6(0-35-0) | ปีที่ 4 ภาคการศึกษาที่ 2 (หน้า 35)
+ภาคนั้นรวม 6 หน่วยกิตตามแผนในเล่ม (ในแผนปกติภาคเดียวกันรวม 12 หน่วยกิต)</t>
+        </is>
+      </c>
+      <c r="H653" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 35</t>
+        </is>
+      </c>
+      <c r="I653" s="39" t="inlineStr">
+        <is>
+          <t>Structured SQL (ตารางแผนปกติ/แผนสหกิจ) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J653" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K653" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L653" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M653" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_coop.json)</t>
+        </is>
+      </c>
+      <c r="N653" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O653" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="654" ht="14.25" customHeight="1" s="36">
+      <c r="A654" s="37" t="inlineStr">
+        <is>
+          <t>QC7</t>
+        </is>
+      </c>
+      <c r="B654" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C654" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D654" s="39" t="inlineStr">
+        <is>
+          <t>เก็บครบ 129 หน่วยกิตพอดี เกรดเฉลี่ยสะสม 2.00 พอดี จบได้ไหม</t>
+        </is>
+      </c>
+      <c r="E654" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F654" s="39" t="inlineStr">
+        <is>
+          <t>จบได้ (ครบหน่วยกิตและไม่ต่ำกว่า 2.00)</t>
+        </is>
+      </c>
+      <c r="G654" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: จบได้ตามเกณฑ์หน่วยกิตและเกรด (ถ้าผ่านเงื่อนไขอื่นครบ)
+หลักสูตร IT 2565 (ปริญญาตรี) ต้องเรียนครบไม่น้อยกว่า 129 หน่วยกิต (หน้า 6)
+- หน่วยกิต: เก็บได้ 129 หน่วยกิต → ครบเกณฑ์ 129 หน่วยกิต
+- เกรดเฉลี่ยสะสม 2.00 → ผ่านเกณฑ์ขั้นต่ำ 2.00 (ข้อ 34)
+- เงื่อนไขอื่นตามข้อ 34: สอบผ่านทุกรายวิชาตามโครงสร้างหลักสูตร และผ่านการสอบภาษาอังกฤษ (English Exit exam)</t>
+        </is>
+      </c>
+      <c r="H654" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 6, 88</t>
+        </is>
+      </c>
+      <c r="I654" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวม + เกรดขั้นต่ำ ข้อ 34) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J654" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K654" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L654" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M654" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N654" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O654" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="655" ht="14.25" customHeight="1" s="36">
+      <c r="A655" s="37" t="inlineStr">
+        <is>
+          <t>QC8</t>
+        </is>
+      </c>
+      <c r="B655" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C655" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D655" s="39" t="inlineStr">
+        <is>
+          <t>ตอนนี้มี 130 หน่วยกิต เกรดเฉลี่ย 3.10 จบได้ยัง</t>
+        </is>
+      </c>
+      <c r="E655" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F655" s="39" t="inlineStr">
+        <is>
+          <t>ยังไม่ได้ ต้องครบ 132 ขาด 2</t>
+        </is>
+      </c>
+      <c r="G655" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ยังจบไม่ได้
+หลักสูตร DSBA 2565 (ปริญญาตรี) ต้องเรียนครบไม่น้อยกว่า 132 หน่วยกิต (หน้า 2)
+- หน่วยกิต: เก็บได้ 130 หน่วยกิต → ยังขาดอีก 2 หน่วยกิต (ต้องครบ 132)
+- เกรดเฉลี่ยสะสม 3.10 → ผ่านเกณฑ์ขั้นต่ำ 2.00 (ข้อ 34)
+- เงื่อนไขอื่นตามข้อ 34: สอบผ่านทุกรายวิชาตามโครงสร้างหลักสูตร และผ่านการสอบภาษาอังกฤษ (English Exit exam)</t>
+        </is>
+      </c>
+      <c r="H655" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 2, 88</t>
+        </is>
+      </c>
+      <c r="I655" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวม + เกรดขั้นต่ำ ข้อ 34) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J655" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K655" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L655" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M655" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N655" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O655" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="656" ht="14.25" customHeight="1" s="36">
+      <c r="A656" s="37" t="inlineStr">
+        <is>
+          <t>QC9</t>
+        </is>
+      </c>
+      <c r="B656" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C656" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D656" s="39" t="inlineStr">
+        <is>
+          <t>จบด้วยเกรดเฉลี่ย 3.75 พอดี จะได้เกียรตินิยมอันดับ 1 เหรียญทองไหม</t>
+        </is>
+      </c>
+      <c r="E656" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F656" s="39" t="inlineStr">
+        <is>
+          <t>ได้ (&gt;= 3.75)</t>
+        </is>
+      </c>
+      <c r="G656" s="39" t="inlineStr">
+        <is>
+          <t>ปริญญาเกียรตินิยม — ข้อ 36 ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 88, 89
+(ข้อบังคับของสถาบัน ใช้กับทุกหลักสูตรปริญญาตรี)
+- เกียรตินิยมอันดับหนึ่งและเหรียญทอง: ค่าระดับคะแนนเฉลี่ยสะสมตามโครงสร้างหลักสูตรสูงสุดในกลุ่มผู้สำเร็จการศึกษาปีเดียวกันของหลักสูตร และค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.75 และต้องไม่เทียบโอนผลการเรียนจากสถาบันอื่น
+- เกียรตินิยมอันดับหนึ่ง: ค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.50
+- เกียรตินิยมอันดับสอง: ค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.25
+- กรณีโอนผลการเรียนจากสถาบันอื่น ทุกรายวิชาต้องได้ไม่ต่ำกว่า B หรือ S และต้องเรียนในหลักสูตรของสถาบันไม่น้อยกว่า 2 ใน 3 ของหน่วยกิตรวม
+- เงื่อนไขทั่วไป (ข้อ 36.1): เรียนไม่เกินระยะเวลาตามแผนการศึกษา · ไม่มีรายวิชาใดได้ F หรือ U · ไม่เคยเรียนซ้ำเพื่อเปลี่ยนเกรด · ไม่เคยลาพักเพราะไม่ลงทะเบียนตามกำหนด และไม่เคยถูกลงโทษทางวินัย</t>
+        </is>
+      </c>
+      <c r="H656" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 88, 89</t>
+        </is>
+      </c>
+      <c r="I656" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J656" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K656" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L656" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M656" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N656" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O656" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="657" ht="14.25" customHeight="1" s="36">
+      <c r="A657" s="37" t="inlineStr">
+        <is>
+          <t>QC10</t>
+        </is>
+      </c>
+      <c r="B657" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C657" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D657" s="39" t="inlineStr">
+        <is>
+          <t>เกรดเฉลี่ยสะสมตอนจบ 3.20 ยังได้เกียรตินิยมอยู่ไหม</t>
+        </is>
+      </c>
+      <c r="E657" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F657" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ได้ อันดับ 2 ต้อง &gt;= 3.25</t>
+        </is>
+      </c>
+      <c r="G657" s="39" t="inlineStr">
+        <is>
+          <t>ปริญญาเกียรตินิยม — ข้อ 36 ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 88, 89
+(ข้อบังคับของสถาบัน ใช้กับทุกหลักสูตรปริญญาตรี)
+- เกียรตินิยมอันดับหนึ่งและเหรียญทอง: ค่าระดับคะแนนเฉลี่ยสะสมตามโครงสร้างหลักสูตรสูงสุดในกลุ่มผู้สำเร็จการศึกษาปีเดียวกันของหลักสูตร และค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.75 และต้องไม่เทียบโอนผลการเรียนจากสถาบันอื่น
+- เกียรตินิยมอันดับหนึ่ง: ค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.50
+- เกียรตินิยมอันดับสอง: ค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.25
+- กรณีโอนผลการเรียนจากสถาบันอื่น ทุกรายวิชาต้องได้ไม่ต่ำกว่า B หรือ S และต้องเรียนในหลักสูตรของสถาบันไม่น้อยกว่า 2 ใน 3 ของหน่วยกิตรวม
+- เงื่อนไขทั่วไป (ข้อ 36.1): เรียนไม่เกินระยะเวลาตามแผนการศึกษา · ไม่มีรายวิชาใดได้ F หรือ U · ไม่เคยเรียนซ้ำเพื่อเปลี่ยนเกรด · ไม่เคยลาพักเพราะไม่ลงทะเบียนตามกำหนด และไม่เคยถูกลงโทษทางวินัย</t>
+        </is>
+      </c>
+      <c r="H657" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 88, 89</t>
+        </is>
+      </c>
+      <c r="I657" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J657" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K657" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L657" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M657" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N657" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O657" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="658" ht="14.25" customHeight="1" s="36">
+      <c r="A658" s="37" t="inlineStr">
+        <is>
+          <t>QC11</t>
+        </is>
+      </c>
+      <c r="B658" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C658" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D658" s="39" t="inlineStr">
+        <is>
+          <t>ย้ายจาก IT ไป DSBA ต้องเรียนรวมกี่หน่วยกิต มากกว่าของเดิมกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E658" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F658" s="39" t="inlineStr">
+        <is>
+          <t>DSBA 132 มากกว่า IT 129 อยู่ 3</t>
+        </is>
+      </c>
+      <c r="G658" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ต่างกัน 3 หน่วยกิต (DSBA 2565 (ปริญญาตรี) มากกว่า IT 2565 (ปริญญาตรี))
+- IT 2565 (ปริญญาตรี): ไม่น้อยกว่า 129 หน่วยกิต (หน้า 6)
+- DSBA 2565 (ปริญญาตรี): ไม่น้อยกว่า 132 หน่วยกิต (หน้า 2)</t>
+        </is>
+      </c>
+      <c r="H658" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 6, 2</t>
+        </is>
+      </c>
+      <c r="I658" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมข้ามหลักสูตร) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J658" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K658" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L658" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M658" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N658" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O658" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="659" ht="14.25" customHeight="1" s="36">
+      <c r="A659" s="37" t="inlineStr">
+        <is>
+          <t>QC12</t>
+        </is>
+      </c>
+      <c r="B659" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C659" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D659" s="39" t="inlineStr">
+        <is>
+          <t>เทอมแรกได้เกรดเฉลี่ย 1.80 จะเกิดอะไรขึ้น</t>
+        </is>
+      </c>
+      <c r="E659" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F659" s="39" t="inlineStr">
+        <is>
+          <t>ถูกภาคทัณฑ์ (ต่ำกว่า 2.00)</t>
+        </is>
+      </c>
+      <c r="G659" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: เกรดเฉลี่ย 1.80 ต่ำกว่า 2.00 → ถูกภาคทัณฑ์ (ข้อ 31) ถ้าภาคถัดไปเกรดเฉลี่ยประจำภาคยังต่ำกว่า 2.00 จะพ้นสภาพ (ข้อ 43.10)
+เมื่อเกรดเฉลี่ยต่ำกว่าเกณฑ์ — ภาคทัณฑ์ (ข้อ 31) และพ้นสภาพ (ข้อ 43) ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 87, 94, 95
+(ข้อบังคับของสถาบัน ใช้กับทุกหลักสูตรปริญญาตรี)
+- ค่าระดับคะแนนเฉลี่ยสะสมต่ำกว่า 2.00: ถูกภาคทัณฑ์ และพ้นภาคทัณฑ์เมื่อกลับมาไม่ต่ำกว่า 2.00 (นับรวมภาคพิเศษ)
+- ระหว่างภาคทัณฑ์ ถ้าค่าระดับคะแนนเฉลี่ยประจำภาคถัดไปต่ำกว่า 2.00: พ้นสภาพนักศึกษา (ข้อ 43.10)
+- ค่าระดับคะแนนเฉลี่ยสะสมต่ำกว่า 1.00: พ้นสภาพนักศึกษา (ข้อ 43.11)
+- สำเร็จการศึกษาได้ต้องมีค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 2.00 (ข้อ 34)</t>
+        </is>
+      </c>
+      <c r="H659" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 87, 94, 95</t>
+        </is>
+      </c>
+      <c r="I659" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J659" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="K659" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L659" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M659" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก ข้อบังคับ ป.ตรี (AIT 2566 ภาคผนวก หน้า 87, 94-95))</t>
+        </is>
+      </c>
+      <c r="N659" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O659" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="660" ht="14.25" customHeight="1" s="36">
+      <c r="A660" s="37" t="inlineStr">
+        <is>
+          <t>QC13</t>
+        </is>
+      </c>
+      <c r="B660" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C660" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D660" s="39" t="inlineStr">
+        <is>
+          <t>ติดโปรอยู่ แล้วเทอมถัดมาได้เกรดเฉลี่ยประจำภาค 1.90 จะโดนรีไทร์ไหม</t>
+        </is>
+      </c>
+      <c r="E660" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F660" s="39" t="inlineStr">
+        <is>
+          <t>พ้นสภาพ (ข้อ 43.10)</t>
+        </is>
+      </c>
+      <c r="G660" s="39" t="inlineStr">
+        <is>
+          <t>การภาคทัณฑ์ — ข้อ 31 ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 87
+(ข้อบังคับของสถาบัน ใช้กับทุกหลักสูตรปริญญาตรี)
+- นักศึกษาที่ได้ค่าระดับคะแนนเฉลี่ยสะสมต่ำกว่า 2.00 ต้องถูกภาคทัณฑ์
+- จะพ้นภาคทัณฑ์เมื่อค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 2.00 (นับรวมภาคการศึกษาพิเศษด้วย)
+- ถ้าระหว่างภาคทัณฑ์ได้ค่าระดับคะแนนเฉลี่ยประจำภาคถัดไปต่ำกว่า 2.00 จะพ้นสภาพนักศึกษา (ข้อ 43.10)</t>
+        </is>
+      </c>
+      <c r="H660" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 87</t>
+        </is>
+      </c>
+      <c r="I660" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J660" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K660" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L660" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M660" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก ข้อบังคับ ป.ตรี (AIT 2566 ภาคผนวก หน้า 87, 94-95))</t>
+        </is>
+      </c>
+      <c r="N660" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O660" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="661" ht="14.25" customHeight="1" s="36">
+      <c r="A661" s="37" t="inlineStr">
+        <is>
+          <t>QC14</t>
+        </is>
+      </c>
+      <c r="B661" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C661" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D661" s="39" t="inlineStr">
+        <is>
+          <t>เกรดเฉลี่ยสะสม 0.95 ยังเรียนต่อได้ไหม</t>
+        </is>
+      </c>
+      <c r="E661" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F661" s="39" t="inlineStr">
+        <is>
+          <t>พ้นสภาพ (ต่ำกว่า 1.00 ข้อ 43.11)</t>
+        </is>
+      </c>
+      <c r="G661" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ได้  
+เกรดเฉลี่ยสะสม 0.95 ต่ำกว่าเกณฑ์ 1.00 ตามข้อ 43.11 แห่งข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (หน้า 95) ทำให้พ้นสภาพนักศึกษาทันที ไม่สามารถเรียนต่อได้  
+ข้อมูลอ้างอิง: ข้อ 43.11 (ภาคผนวกในเล่ม มคอ.2 AIT 2566)</t>
+        </is>
+      </c>
+      <c r="H661" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 87, 94, 95</t>
+        </is>
+      </c>
+      <c r="I661" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) → Typhoon เรียบเรียง</t>
+        </is>
+      </c>
+      <c r="J661" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="K661" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L661" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M661" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก ข้อบังคับ ป.ตรี (AIT 2566 ภาคผนวก หน้า 87, 94-95))</t>
+        </is>
+      </c>
+      <c r="N661" s="39" t="inlineStr">
+        <is>
+          <t>1.29s</t>
+        </is>
+      </c>
+      <c r="O661" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="662" ht="14.25" customHeight="1" s="36">
+      <c r="A662" s="37" t="inlineStr">
+        <is>
+          <t>QC15</t>
+        </is>
+      </c>
+      <c r="B662" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C662" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D662" s="39" t="inlineStr">
+        <is>
+          <t>เหลืออีก 9 หน่วยกิตจะจบ ลงซัมเมอร์เทอมเดียวให้ครบเลยได้ไหม</t>
+        </is>
+      </c>
+      <c r="E662" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่) — ชุดที่ระบบไม่เคยเห็น รอบ 7 (ยาก/ท้าทาย แบบใหม่)</t>
+        </is>
+      </c>
+      <c r="F662" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ภาคฤดูร้อนลงได้ไม่เกิน 9</t>
+        </is>
+      </c>
+      <c r="G662" s="39" t="inlineStr">
+        <is>
+          <t>ได้  
+นักศึกษาชั้นปีสุดท้ายที่เหลือรายวิชาไม่ถึง 9 หน่วยกิตสามารถลงทะเบียนเพิ่มได้ถึง 27 หน่วยกิตในภาคการศึกษาปกติหรือภาคพิเศษ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 โดยวิชาที่เรียนในภาคฤดูร้อน (ซัมเมอร์เทอม) สามารถลงทะเบียนได้ไม่เกิน 9 หน่วยกิต แต่หากเป็นวิชาฝึกงาน ห้ามลงวิชาอื่นในภาคเดียวกัน ดังนั้นหากวิชาที่เหลือเป็นวิชาทั่วไปหรือวิชาเลือกที่ไม่ใช่ฝึกงาน สามารถลงได้ในซัมเมอร์เทอมเพื่อให้ครบ 9 หน่วยกิตได้</t>
+        </is>
+      </c>
+      <c r="H662" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 82</t>
+        </is>
+      </c>
+      <c r="I662" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) → Typhoon เรียบเรียง</t>
+        </is>
+      </c>
+      <c r="J662" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K662" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L662" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M662" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก ข้อบังคับ ป.ตรี (AIT 2566 ภาคผนวก หน้า 85))</t>
+        </is>
+      </c>
+      <c r="N662" s="39" t="inlineStr">
+        <is>
+          <t>2.04s</t>
+        </is>
+      </c>
+      <c r="O662" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
     <row r="663" ht="14.25" customHeight="1" s="36"/>
     <row r="664" ht="14.25" customHeight="1" s="36"/>
     <row r="665" ht="14.25" customHeight="1" s="36"/>

</xml_diff>

<commit_message>
feat(query): compare a year's two semesters, whole-year and cumulative plan credits with what remains, two courses' combined credits, all-level prerequisite counts, final-year 27-credit exception; hard/challenge unseen rounds 8-9; tester 705 rows
</commit_message>
<xml_diff>
--- a/docs/tester.xlsx
+++ b/docs/tester.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O662"/>
+  <dimension ref="A1:O706"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10" customWidth="1" style="36" min="1" max="1"/>
@@ -756,7 +756,7 @@
       </c>
       <c r="N2" s="13" t="inlineStr">
         <is>
-          <t>0.03s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O2" s="21" t="inlineStr">
@@ -1340,12 +1340,12 @@
       </c>
       <c r="N9" s="25" t="inlineStr">
         <is>
-          <t>0.62s</t>
+          <t>7.79s</t>
         </is>
       </c>
       <c r="O9" s="21" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="N10" s="13" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O10" s="21" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="N11" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O11" s="21" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="N12" s="13" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>4.63s</t>
         </is>
       </c>
       <c r="O12" s="21" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="N13" s="25" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>3.12s</t>
         </is>
       </c>
       <c r="O13" s="21" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="N14" s="13" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.80s</t>
         </is>
       </c>
       <c r="O14" s="21" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="N15" s="25" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="O15" s="21" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="N20" s="13" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O20" s="21" t="inlineStr">
@@ -2395,7 +2395,7 @@
       <c r="G21" s="34" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาสามารถเรียนวิชาที่เกี่ยวข้องกับฐานข้อมูลในปีที่ 4 ได้ เนื่องจากมีวิชาบังคับก่อนหน้า เช่น 06066300 แนวคิดระบบฐานข้อมูล (ปี 2 ภาค 1) และ 06026212 การสร้างคลังข้อมูล (ปี 3 ภาค 1) ซึ่งเป็นพื้นฐานจำเป็น วิชาที่เกี่ยวข้องในปี 4 ได้แก่ 06026246 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 และ 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 2 ที่จัดสอนในภาคการศึกษาที่ 1 ปีที่ 4 ประเภทวิชาบังคับในกลุ่มวิชาเลือกเฉพาะแขนง ตามหลักสูตร DSBA 2565</t>
+นักศึกษาสามารถเรียนวิชาฐานข้อมูลในปีที่ 4 ได้ เนื่องจากมีวิชาบังคับในกลุ่มวิชาเลือกเฉพาะแขนง เช่น 06026246 หัวข้อพิเศษทางวิศวกรรมข้อมูล 1 และ 06026247 หัวข้อพิเศษทางวิศวกรรมข้อมูล 2 ซึ่งจัดสอนในภาคการศึกษาที่ 2 ปีที่ 4 โดยมีวิชาบังคับก่อนหน้าคือ 06066300 แนวคิดระบบฐานข้อมูล (ปีที่ 2 ภาคการศึกษาที่ 1) และ 06026212 การสร้างคลังข้อมูล (ปีที่ 3 ภาคการศึกษาที่ 1) ที่ครอบคลุมเนื้อหาพื้นฐานด้านฐานข้อมูลอย่างเพียงพอ</t>
         </is>
       </c>
       <c r="H21" s="34" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="N21" s="13" t="inlineStr">
         <is>
-          <t>2.88s</t>
+          <t>1.90s</t>
         </is>
       </c>
       <c r="O21" s="21" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="N23" s="13" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.26s</t>
         </is>
       </c>
       <c r="O23" s="21" t="inlineStr">
@@ -2801,11 +2801,15 @@
       </c>
       <c r="G25" s="34" t="inlineStr">
         <is>
-          <t>ใช่ หลักสูตรวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปีที่ 3 มีการเลือกแขนง (หรือที่เรียกว่า "กลุ่มวิชา") ให้เลือก โดยมี 3 แขนง ดังนี้:
-- กลุ่มวิทยาการข้อมูล (Data Science)  
-- กลุ่มการวิเคราะห์เชิงสถิติ (Statistical Analytics)  
-- กลุ่มวิศวกรรมข้อมูล (Data Engineering)  
-[3][4][6]</t>
+          <t>ใช่ หลักสูตรวิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ (DSBA) ปีที่ 3 มีการเลือกแขนง (หรือที่เรียกว่า "กลุ่มวิชา") ซึ่งแบ่งออกเป็น 3 แขนง ดังนี้:
+- วิทยาการข้อมูล (Data Science)  
+- การวิเคราะห์เชิงสถิติ (Statistical Analysis)  
+- วิศวกรรมข้อมูล (Data Engineering)  
+แต่ละแขนงมีรายวิชาเลือกที่เกี่ยวข้อง ได้แก่:
+- วิชาเลือกกลุ่มวิทยาการข้อมูล 1–4 (ELECTIVE IN DATA SCIENCE 1–4)  
+- วิชาเลือกกลุ่มการวิเคราะห์เชิงสถิติ 1–4 (ELECTIVE IN STATISTICAL ANALYTICS 1–4)  
+- วิชาเลือกกลุ่มวิศวกรรมข้อมูล 1–4 (ELECTIVE IN DATA ENGINEERING 1–4)  
+[3], [4], [6]</t>
         </is>
       </c>
       <c r="H25" s="34" t="inlineStr">
@@ -2838,7 +2842,7 @@
       </c>
       <c r="N25" s="13" t="inlineStr">
         <is>
-          <t>1.64s</t>
+          <t>2.33s</t>
         </is>
       </c>
       <c r="O25" s="21" t="inlineStr">
@@ -2880,9 +2884,9 @@
       </c>
       <c r="G26" s="34" t="inlineStr">
         <is>
-          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวมน้อยกว่า IT 2560 อยู่ 1 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูลแทนการเลือกแขนงวิชาเดิม
-2. หลักสูตร IT 2560 มีหน่วยกิตรวม 130 หน่วยกิต (มคอ.2 IT 2560 หน้า 18) ขณะที่ IT 2565 มี 129 หน่วยกิต (มคอ.2 IT 2565 หน้า 6) ลดลง 1 หน่วยกิต ซึ่งสะท้อนจากการปรับโครงสร้างกลุ่มวิชาเฉพาะด้านและวิชาเลือก โดยเฉพาะการเปลี่ยนจาก "แขนงวิชา" มาเป็น "โมดูลอาชีพ" 3 โมดูล (M1-M3) ที่มีความยืดหยุ่นในการเลือกวิชา และลดหน่วยกิตในกลุ่มวิชาบังคับเฉพาะแขนงจาก 30 เป็น 15 หน่วยกิต (ข้อมูลจาก [3], [4], [8])
-3. อ้างข้อมูลจากหลักฐาน: หน่วยกิตรวม (IT 2560 vs IT 2565), ประเภทวิชา (บังคับ/เลือก), ภาค/ปีที่เปิดสอน (IT 2560 เริ่มภาค 1/2560, IT 2565 เริ่มภาค 1/2565), โครงสร้างแขนงวิชา (เปลี่ยนจาก "แขนงวิชา" เป็น "โมดูลอาชีพ")</t>
+          <t>1. หลักสูตร IT 2565 มีหน่วยกิตรวม 129 หน่วยกิต ลดลง 1 หน่วยกิตจาก IT 2560 ที่มี 130 หน่วยกิต และเปลี่ยนโครงสร้างแขนงวิชาเป็น "โมดูลอาชีพ" 3 โมดูลแทนการเลือกแขนงวิชาเดิม
+2. หลักสูตร IT 2565 ปรับโครงสร้างให้เน้นความรู้เชิงลึกผ่าน "โมดูลอาชีพ" 3 โมดูล (Full-Stack Web Developer, Network/System Engineer, Game Developer) แทนการเลือก "แขนงวิชา" 3 แขนงใน IT 2560 พร้อมเพิ่มหน่วยกิตวิชาเลือกทางเทคโนโลยีสารสนเทศจาก 6 เป็น 9 หน่วยกิต และย้ายรายวิชาบางวิชาเข้าโมดูลเพื่อความสอดคล้องกับความต้องการตลาดแรงงาน
+3. อ้างข้อมูลจาก: หน่วยกิตรวม (มคอ.2 IT 2560 หน้า 18, IT 2565 หน้า 6), โครงสร้างหลักสูตร (IT 2565 หน้า 371, 374, 376, 378), การปรับโครงสร้าง (IT 2565 หน้า 370, 374), ประเภทวิชา (บังคับ/เลือก) และการเปลี่ยนแปลงจาก "แขนงวิชา" เป็น "โมดูลอาชีพ" (IT 2565 หน้า 370, 376, 378)</t>
         </is>
       </c>
       <c r="H26" s="34" t="inlineStr">
@@ -2915,7 +2919,7 @@
       </c>
       <c r="N26" s="13" t="inlineStr">
         <is>
-          <t>4.90s</t>
+          <t>3.43s</t>
         </is>
       </c>
       <c r="O26" s="21" t="inlineStr">
@@ -3067,7 +3071,7 @@
       <c r="M28" s="34" t="n"/>
       <c r="N28" s="13" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.40s</t>
         </is>
       </c>
       <c r="O28" s="21" t="inlineStr">
@@ -3143,7 +3147,7 @@
       </c>
       <c r="N29" s="25" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.17s</t>
         </is>
       </c>
       <c r="O29" s="21" t="inlineStr">
@@ -3404,7 +3408,7 @@
       </c>
       <c r="N32" s="13" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O32" s="21" t="inlineStr">
@@ -3484,7 +3488,7 @@
       </c>
       <c r="N33" s="25" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.27s</t>
         </is>
       </c>
       <c r="O33" s="21" t="inlineStr">
@@ -3632,7 +3636,7 @@
       <c r="M35" s="35" t="n"/>
       <c r="N35" s="25" t="inlineStr">
         <is>
-          <t>0.52s</t>
+          <t>0.54s</t>
         </is>
       </c>
       <c r="O35" s="21" t="inlineStr">
@@ -3710,7 +3714,7 @@
       </c>
       <c r="N36" s="13" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O36" s="21" t="inlineStr">
@@ -3753,16 +3757,20 @@
       <c r="G37" s="35" t="inlineStr">
         <is>
           <t>วิชาที่เกี่ยวข้องกับ "machine learning" — หลักสูตร AIT
-■ AIT 2566 — 7 วิชา รวม 17 หน่วยกิต
+■ AIT 2566 — 9 วิชา รวม 23 หน่วยกิต
   - 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING)
       หน่วยกิต 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
   - 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING)
       หน่วยกิต 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1
   - 06046414 การประมวลผลภาษาธรรมชาติด้วยการเรียนรู้เชิงลึก (NATURAL LANGUAGE PROCESSING WITH DEEP LEARNING)
       หน่วยกิต 3(3-0-6) | ปีที่ 3 ภาคการศึกษาที่ 1
+  - 06046415 การประมวลผลสัญญาณ (SIGNAL PROCESSING)
+      หน่วยกิต 3(3-0-6) | ปีที่ 3 ภาคการศึกษาที่ 1
   - 06046416 การเรียนรู้เชิงลึกสำหรับคอมพิวเตอร์วิทัศน์ (DEEP LEARNING FOR COMPUTER VISION)
       หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
   - 06046419 การเรียนรู้แบบเสริมกำลัง (REINFORCEMENT LEARNING)
+      หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
+  - 90642113 หุ่นยนต์และปัญญาประดิษฐ์ (ROBOTICS A)
       หน่วยกิต 3(3-0-6) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
   - 90964204 สารสนเทศเพื่อการเรียนรู้ (INFORMATION FOR LEARNING)
       หน่วยกิต 1(0-2-1) | ไม่ระบุชั้นปี (วิชาเลือก/วิชาในหมวดเลือก)
@@ -3800,7 +3808,7 @@
       </c>
       <c r="N37" s="25" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.36s</t>
         </is>
       </c>
       <c r="O37" s="21" t="inlineStr">
@@ -3912,7 +3920,7 @@
       </c>
       <c r="N38" s="13" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.28s</t>
         </is>
       </c>
       <c r="O38" s="21" t="inlineStr">
@@ -4004,7 +4012,7 @@
       </c>
       <c r="N39" s="25" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.40s</t>
         </is>
       </c>
       <c r="O39" s="21" t="inlineStr">
@@ -4341,7 +4349,7 @@
       <c r="M43" s="35" t="n"/>
       <c r="N43" s="25" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O43" s="21" t="inlineStr">
@@ -4417,7 +4425,7 @@
       </c>
       <c r="N44" s="13" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.25s</t>
         </is>
       </c>
       <c r="O44" s="21" t="inlineStr">
@@ -4650,7 +4658,7 @@
       </c>
       <c r="N47" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O47" s="21" t="inlineStr">
@@ -4898,7 +4906,7 @@
       </c>
       <c r="N50" s="13" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.17s</t>
         </is>
       </c>
       <c r="O50" s="21" t="inlineStr">
@@ -6645,7 +6653,7 @@
       <c r="M70" s="34" t="n"/>
       <c r="N70" s="13" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O70" s="21" t="inlineStr">
@@ -6723,7 +6731,7 @@
       </c>
       <c r="N71" s="25" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O71" s="21" t="inlineStr">
@@ -6801,7 +6809,7 @@
       </c>
       <c r="N72" s="13" t="inlineStr">
         <is>
-          <t>0.08s</t>
+          <t>0.18s</t>
         </is>
       </c>
       <c r="O72" s="21" t="inlineStr">
@@ -7200,7 +7208,7 @@
       </c>
       <c r="N77" s="25" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O77" s="21" t="inlineStr">
@@ -7284,7 +7292,7 @@
       </c>
       <c r="N78" s="13" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O78" s="21" t="inlineStr">
@@ -7393,7 +7401,7 @@
       </c>
       <c r="N79" s="25" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O79" s="21" t="inlineStr">
@@ -7549,7 +7557,7 @@
       </c>
       <c r="N81" s="25" t="inlineStr">
         <is>
-          <t>0.08s</t>
+          <t>0.07s</t>
         </is>
       </c>
       <c r="O81" s="21" t="inlineStr">
@@ -7736,7 +7744,7 @@
       </c>
       <c r="N83" s="25" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O83" s="21" t="inlineStr">
@@ -11809,7 +11817,7 @@
       </c>
       <c r="N135" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O135" s="41" t="inlineStr">
@@ -12046,7 +12054,7 @@
       </c>
       <c r="N138" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O138" s="41" t="inlineStr">
@@ -12204,7 +12212,7 @@
       </c>
       <c r="N140" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O140" s="41" t="inlineStr">
@@ -12362,7 +12370,7 @@
       </c>
       <c r="N142" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O142" s="41" t="inlineStr">
@@ -12520,7 +12528,7 @@
       </c>
       <c r="N144" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O144" s="41" t="inlineStr">
@@ -12678,7 +12686,7 @@
       </c>
       <c r="N146" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O146" s="41" t="inlineStr">
@@ -12757,7 +12765,7 @@
       </c>
       <c r="N147" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O147" s="41" t="inlineStr">
@@ -13309,7 +13317,7 @@
       </c>
       <c r="N154" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O154" s="41" t="inlineStr">
@@ -13467,7 +13475,7 @@
       </c>
       <c r="N156" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O156" s="41" t="inlineStr">
@@ -14245,7 +14253,7 @@
       </c>
       <c r="N166" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O166" s="41" t="inlineStr">
@@ -14821,7 +14829,7 @@
       </c>
       <c r="N173" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O173" s="41" t="inlineStr">
@@ -17462,7 +17470,7 @@
       </c>
       <c r="N206" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O206" s="41" t="inlineStr">
@@ -17539,7 +17547,7 @@
       </c>
       <c r="N207" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O207" s="41" t="inlineStr">
@@ -18125,7 +18133,7 @@
       </c>
       <c r="N214" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O214" s="41" t="inlineStr">
@@ -19476,7 +19484,7 @@
       </c>
       <c r="N231" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O231" s="41" t="inlineStr">
@@ -19556,7 +19564,7 @@
       </c>
       <c r="N232" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O232" s="41" t="inlineStr">
@@ -20043,7 +20051,7 @@
       </c>
       <c r="N238" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O238" s="41" t="inlineStr">
@@ -20120,7 +20128,7 @@
       </c>
       <c r="N239" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O239" s="41" t="inlineStr">
@@ -20197,7 +20205,7 @@
       </c>
       <c r="N240" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O240" s="41" t="inlineStr">
@@ -20274,7 +20282,7 @@
       </c>
       <c r="N241" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O241" s="41" t="inlineStr">
@@ -20351,7 +20359,7 @@
       </c>
       <c r="N242" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O242" s="41" t="inlineStr">
@@ -21051,7 +21059,7 @@
       </c>
       <c r="N251" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.03s</t>
         </is>
       </c>
       <c r="O251" s="41" t="inlineStr">
@@ -21393,7 +21401,7 @@
       </c>
       <c r="N255" s="39" t="inlineStr">
         <is>
-          <t>0.04s</t>
+          <t>0.03s</t>
         </is>
       </c>
       <c r="O255" s="41" t="inlineStr">
@@ -21475,7 +21483,7 @@
       </c>
       <c r="N256" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O256" s="41" t="inlineStr">
@@ -21558,7 +21566,7 @@
       </c>
       <c r="N257" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O257" s="41" t="inlineStr">
@@ -21715,7 +21723,7 @@
       </c>
       <c r="N259" s="39" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.11s</t>
         </is>
       </c>
       <c r="O259" s="41" t="inlineStr">
@@ -22742,7 +22750,7 @@
       </c>
       <c r="N272" s="39" t="inlineStr">
         <is>
-          <t>0.04s</t>
+          <t>0.05s</t>
         </is>
       </c>
       <c r="O272" s="41" t="inlineStr">
@@ -25317,7 +25325,7 @@
       </c>
       <c r="N305" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O305" s="41" t="inlineStr">
@@ -25632,7 +25640,7 @@
       </c>
       <c r="N309" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O309" s="41" t="inlineStr">
@@ -27762,7 +27770,7 @@
       </c>
       <c r="N336" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O336" s="41" t="inlineStr">
@@ -27841,7 +27849,7 @@
       </c>
       <c r="N337" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O337" s="41" t="inlineStr">
@@ -28633,7 +28641,7 @@
       </c>
       <c r="N347" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O347" s="41" t="inlineStr">
@@ -28710,7 +28718,7 @@
       </c>
       <c r="N348" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O348" s="41" t="inlineStr">
@@ -28787,7 +28795,7 @@
       </c>
       <c r="N349" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O349" s="41" t="inlineStr">
@@ -29495,7 +29503,7 @@
       </c>
       <c r="N358" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O358" s="41" t="inlineStr">
@@ -29697,8 +29705,7 @@
       </c>
       <c r="G361" s="39" t="inlineStr">
         <is>
-          <t>ได้  
-นักศึกษาชั้นปีสุดท้ายที่เหลือรายวิชาไม่ถึง 9 หน่วยกิต หรือต้องลงเกิน 22 หน่วยกิตเพื่อสำเร็จการศึกษา สามารถลงทะเบียนได้สูงสุดไม่เกิน 27 หน่วยกิต โดยต้องได้รับอนุมัติจากสภาวิชาการ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 ซึ่งระบุไว้ชัดเจนสำหรับกรณีปีสุดท้าย</t>
+          <t>ได้ — นักศึกษาชั้นปีสุดท้ายที่เหลือรายวิชาไม่ถึง 9 หน่วยกิต หรือต้องลงเกิน 22 หน่วยกิตเพื่อสำเร็จการศึกษา สามารถลงทะเบียนได้สูงสุด 27 หน่วยกิต โดยต้องได้รับอนุมัติจากสภาวิชาการ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 ประเภทวิชา: บังคับ (สำหรับนักศึกษาที่ต้องการสำเร็จการศึกษา)</t>
         </is>
       </c>
       <c r="H361" s="39" t="inlineStr">
@@ -29731,7 +29738,7 @@
       </c>
       <c r="N361" s="39" t="inlineStr">
         <is>
-          <t>1.51s</t>
+          <t>1.58s</t>
         </is>
       </c>
       <c r="O361" s="41" t="inlineStr">
@@ -29813,7 +29820,7 @@
       </c>
       <c r="N362" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O362" s="41" t="inlineStr">
@@ -30529,7 +30536,7 @@
       </c>
       <c r="N371" s="39" t="inlineStr">
         <is>
-          <t>0.03s</t>
+          <t>0.02s</t>
         </is>
       </c>
       <c r="O371" s="41" t="inlineStr">
@@ -32083,7 +32090,7 @@
       </c>
       <c r="N391" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O391" s="41" t="inlineStr">
@@ -32399,7 +32406,7 @@
       </c>
       <c r="N395" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O395" s="41" t="inlineStr">
@@ -33192,7 +33199,7 @@
       </c>
       <c r="N405" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O405" s="41" t="inlineStr">
@@ -33269,7 +33276,7 @@
       </c>
       <c r="N406" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O406" s="41" t="inlineStr">
@@ -33346,7 +33353,7 @@
       </c>
       <c r="N407" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O407" s="41" t="inlineStr">
@@ -33500,7 +33507,7 @@
       </c>
       <c r="N409" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O409" s="41" t="inlineStr">
@@ -34522,7 +34529,7 @@
       </c>
       <c r="N422" s="39" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="O422" s="41" t="inlineStr">
@@ -36816,7 +36823,7 @@
       </c>
       <c r="N451" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O451" s="41" t="inlineStr">
@@ -36973,7 +36980,7 @@
       </c>
       <c r="N453" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O453" s="41" t="inlineStr">
@@ -37287,7 +37294,7 @@
       </c>
       <c r="N457" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O457" s="41" t="inlineStr">
@@ -37364,7 +37371,7 @@
       </c>
       <c r="N458" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O458" s="41" t="inlineStr">
@@ -37441,7 +37448,7 @@
       </c>
       <c r="N459" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O459" s="41" t="inlineStr">
@@ -40268,7 +40275,7 @@
       </c>
       <c r="N495" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O495" s="41" t="inlineStr">
@@ -41143,7 +41150,7 @@
       </c>
       <c r="N506" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O506" s="41" t="inlineStr">
@@ -41220,7 +41227,7 @@
       </c>
       <c r="N507" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O507" s="41" t="inlineStr">
@@ -42437,7 +42444,7 @@
       </c>
       <c r="N522" s="39" t="inlineStr">
         <is>
-          <t>0.53s</t>
+          <t>0.80s</t>
         </is>
       </c>
       <c r="O522" s="41" t="inlineStr">
@@ -42679,7 +42686,7 @@
       </c>
       <c r="N525" s="39" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.78s</t>
         </is>
       </c>
       <c r="O525" s="41" t="inlineStr">
@@ -43315,7 +43322,7 @@
       </c>
       <c r="N533" s="39" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.10s</t>
         </is>
       </c>
       <c r="O533" s="41" t="inlineStr">
@@ -43624,7 +43631,7 @@
       </c>
       <c r="N537" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O537" s="41" t="inlineStr">
@@ -44172,7 +44179,7 @@
       </c>
       <c r="N544" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O544" s="41" t="inlineStr">
@@ -44409,7 +44416,7 @@
       </c>
       <c r="N547" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O547" s="41" t="inlineStr">
@@ -44488,7 +44495,7 @@
       </c>
       <c r="N548" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O548" s="41" t="inlineStr">
@@ -45258,7 +45265,7 @@
       </c>
       <c r="N557" s="39" t="inlineStr">
         <is>
-          <t>0.01s</t>
+          <t>0.00s</t>
         </is>
       </c>
       <c r="O557" s="41" t="inlineStr">
@@ -46055,7 +46062,7 @@
       </c>
       <c r="N567" s="39" t="inlineStr">
         <is>
-          <t>0.02s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O567" s="41" t="inlineStr">
@@ -46242,7 +46249,7 @@
       </c>
       <c r="N569" s="39" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>1.07s</t>
         </is>
       </c>
       <c r="O569" s="41" t="inlineStr">
@@ -47111,7 +47118,7 @@
       </c>
       <c r="N580" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O580" s="41" t="inlineStr">
@@ -48650,7 +48657,9 @@
       <c r="G600" s="39" t="inlineStr">
         <is>
           <t>ไม่ได้  
-นักศึกษาทั่วไปต้องลงทะเบียนไม่เกิน 22 หน่วยกิตต่อภาคการศึกษาปกติ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 แม้จะเป็นนักศึกษาชั้นปีสุดท้ายก็ตาม แต่ต้องไม่เกิน 27 หน่วยกิต หากมีข้อยกเว้นเฉพาะกรณีที่เหลือรายวิชาไม่ถึง 3 หน่วยกิต หรือต้องลงเพื่อสำเร็จการศึกษา ซึ่งไม่ได้ระบุว่าเป็นกรณีนี้ ดังนั้นการลง 25 หน่วยกิตเกินข้อจำกัดปกติ และไม่มีหลักฐานยืนยันว่าเข้าข่ายข้อยกเว้น</t>
+นักศึกษาทั่วไปต้องลงทะเบียนไม่เกิน 22 หน่วยกิตต่อภาคการศึกษาปกติ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82  
+แม้จะมีข้อยกเว้นสำหรับนักศึกษาชั้นปีสุดท้ายที่อาจลงได้ไม่เกิน 27 หน่วยกิต แต่ต้องมีเหตุผลชัดเจน เช่น เหลือรายวิชาไม่ถึง 3 หน่วยกิต หรือต้องลงเพื่อสำเร็จการศึกษา  
+การลง 25 หน่วยกิตโดยไม่เข้าเงื่อนไขข้อยกเว้นดังกล่าว จึงไม่ได้รับอนุญาตตามข้อบังคับโดยตรง</t>
         </is>
       </c>
       <c r="H600" s="39" t="inlineStr">
@@ -48683,7 +48692,7 @@
       </c>
       <c r="N600" s="39" t="inlineStr">
         <is>
-          <t>2.24s</t>
+          <t>3.51s</t>
         </is>
       </c>
       <c r="O600" s="41" t="inlineStr">
@@ -49387,7 +49396,7 @@
       </c>
       <c r="N609" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O609" s="41" t="inlineStr">
@@ -51003,7 +51012,7 @@
       <c r="G630" s="39" t="inlineStr">
         <is>
           <t>ไม่ได้  
-นักศึกษาต้องลงทะเบียนไม่น้อยกว่า 9 หน่วยกิตในภาคการศึกษาปกติ ตามข้อบังคับสถาบันเทคโนโลยีพระจอมเกล้าเจ้าคุณทหารลาดกระบัง ว่าด้วยการศึกษาระดับปริญญาตรี พ.ศ. 2564 (ภาคผนวก ก) ซึ่งใช้กับหลักสูตรวท.บ. (วิทยาการข้อมูลและการวิเคราะห์เชิงธุรกิจ) คณะเทคโนโลยีสารสนเทศ สจล. ทุกภาคการศึกษาปกติ</t>
+นักศึกษาต้องลงทะเบียนไม่น้อยกว่า 9 หน่วยกิตในภาคการศึกษาปกติ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 ซึ่งเป็นข้อกำหนดบังคับสำหรับทุกหลักสูตรปริญญาตรี ทั้งนี้ ไม่มีข้อยกเว้นสำหรับนักศึกษาชั้นปีที่ 1 หรือภาคเรียนแรกที่สามารถลงทะเบียนต่ำกว่า 9 หน่วยกิตได้</t>
         </is>
       </c>
       <c r="H630" s="39" t="inlineStr">
@@ -51036,7 +51045,7 @@
       </c>
       <c r="N630" s="39" t="inlineStr">
         <is>
-          <t>1.61s</t>
+          <t>3.10s</t>
         </is>
       </c>
       <c r="O630" s="41" t="inlineStr">
@@ -51080,8 +51089,8 @@
         <is>
           <t>ได้  
 นักศึกษาสามารถลงทะเบียนเรียนได้ไม่เกิน 9 หน่วยกิตในภาคการศึกษาพิเศษ (ภาคฤดูร้อน) ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82  
-หากลงฝึกงานในภาคพิเศษ ห้ามลงทะเบียนเรียนรายวิชาอื่นเพิ่มเติมได้  
-ประเภทวิชา: ภาคการศึกษาพิเศษ, ข้อบังคับการลงทะเบียนเรียน</t>
+หากลงรายวิชาฝึกงานในภาคพิเศษ จะไม่สามารถลงวิชาอื่นได้ ตามข้อบังคับเดียวกัน  
+ดังนั้น ถ้าลงฝึกงาน ไม่สามารถลงวิชาอื่นได้ และจำนวนหน่วยกิตสูงสุดที่สามารถลงทะเบียนได้คือ 9 หน่วยกิต (เฉพาะฝึกงาน)</t>
         </is>
       </c>
       <c r="H631" s="39" t="inlineStr">
@@ -51114,7 +51123,7 @@
       </c>
       <c r="N631" s="39" t="inlineStr">
         <is>
-          <t>1.75s</t>
+          <t>2.86s</t>
         </is>
       </c>
       <c r="O631" s="41" t="inlineStr">
@@ -52270,7 +52279,7 @@
       </c>
       <c r="N646" s="39" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>0.01s</t>
         </is>
       </c>
       <c r="O646" s="41" t="inlineStr">
@@ -53411,8 +53420,8 @@
       <c r="G661" s="39" t="inlineStr">
         <is>
           <t>ไม่ได้  
-เกรดเฉลี่ยสะสม 0.95 ต่ำกว่าเกณฑ์ 1.00 ตามข้อ 43.11 แห่งข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (หน้า 95) ทำให้พ้นสภาพนักศึกษาทันที ไม่สามารถเรียนต่อได้  
-ข้อมูลอ้างอิง: ข้อ 43.11 (ภาคผนวกในเล่ม มคอ.2 AIT 2566)</t>
+เกรดเฉลี่ยสะสม 0.95 ต่ำกว่าเกณฑ์ 1.00 ตามข้อ 43.11 ของข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (หน้า 95) ทำให้พ้นสภาพนักศึกษาทันที ไม่สามารถเรียนต่อได้  
+ข้อมูลอ้างอิง: ข้อ 43.11, หน้า 95, ข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566)</t>
         </is>
       </c>
       <c r="H661" s="39" t="inlineStr">
@@ -53445,7 +53454,7 @@
       </c>
       <c r="N661" s="39" t="inlineStr">
         <is>
-          <t>1.29s</t>
+          <t>2.26s</t>
         </is>
       </c>
       <c r="O661" s="41" t="inlineStr">
@@ -53488,7 +53497,7 @@
       <c r="G662" s="39" t="inlineStr">
         <is>
           <t>ได้  
-นักศึกษาชั้นปีสุดท้ายที่เหลือรายวิชาไม่ถึง 9 หน่วยกิตสามารถลงทะเบียนเพิ่มได้ถึง 27 หน่วยกิตในภาคการศึกษาปกติหรือภาคพิเศษ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 โดยวิชาที่เรียนในภาคฤดูร้อน (ซัมเมอร์เทอม) สามารถลงทะเบียนได้ไม่เกิน 9 หน่วยกิต แต่หากเป็นวิชาฝึกงาน ห้ามลงวิชาอื่นในภาคเดียวกัน ดังนั้นหากวิชาที่เหลือเป็นวิชาทั่วไปหรือวิชาเลือกที่ไม่ใช่ฝึกงาน สามารถลงได้ในซัมเมอร์เทอมเพื่อให้ครบ 9 หน่วยกิตได้</t>
+นักศึกษาที่เหลืออีก 9 หน่วยกิตสามารถลงทะเบียนเรียนในภาคฤดูร้อน (ซัมเมอร์เทอม) เพื่อสำเร็จการศึกษาได้ เนื่องจากข้อบังคับอนุญาตให้นักศึกษาชั้นปีสุดท้ายที่เหลือหน่วยกิตน้อยกว่า 9 หน่วยกิต ลงทะเบียนได้ไม่เกิน 27 หน่วยกิต แม้ภาคฤดูร้อนจะจำกัดไว้ที่ไม่เกิน 9 หน่วยกิต แต่หากเป็นรายวิชาที่จำเป็นต้องใช้เพื่อจบการศึกษา สามารถขออนุมัติจากสภาวิชาการได้ ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 82 และหลักสูตร BIT 2565 กำหนดให้ต้องเรียนรวม 90 หน่วยกิต (ไม่รวมสหกิจศึกษา) ซึ่งนักศึกษาที่เหลือ 9 หน่วยกิตจึงสามารถใช้ภาคฤดูร้อนเพื่อจบได้</t>
         </is>
       </c>
       <c r="H662" s="39" t="inlineStr">
@@ -53521,7 +53530,7 @@
       </c>
       <c r="N662" s="39" t="inlineStr">
         <is>
-          <t>2.04s</t>
+          <t>2.95s</t>
         </is>
       </c>
       <c r="O662" s="41" t="inlineStr">
@@ -53530,50 +53539,3457 @@
         </is>
       </c>
     </row>
-    <row r="663" ht="14.25" customHeight="1" s="36"/>
-    <row r="664" ht="14.25" customHeight="1" s="36"/>
-    <row r="665" ht="14.25" customHeight="1" s="36"/>
-    <row r="666" ht="14.25" customHeight="1" s="36"/>
-    <row r="667" ht="14.25" customHeight="1" s="36"/>
-    <row r="668" ht="14.25" customHeight="1" s="36"/>
-    <row r="669" ht="14.25" customHeight="1" s="36"/>
-    <row r="670" ht="14.25" customHeight="1" s="36"/>
-    <row r="671" ht="14.25" customHeight="1" s="36"/>
-    <row r="672" ht="14.25" customHeight="1" s="36"/>
-    <row r="673" ht="14.25" customHeight="1" s="36"/>
-    <row r="674" ht="14.25" customHeight="1" s="36"/>
-    <row r="675" ht="14.25" customHeight="1" s="36"/>
-    <row r="676" ht="14.25" customHeight="1" s="36"/>
-    <row r="677" ht="14.25" customHeight="1" s="36"/>
-    <row r="678" ht="14.25" customHeight="1" s="36"/>
-    <row r="679" ht="14.25" customHeight="1" s="36"/>
-    <row r="680" ht="14.25" customHeight="1" s="36"/>
-    <row r="681" ht="14.25" customHeight="1" s="36"/>
-    <row r="682" ht="14.25" customHeight="1" s="36"/>
-    <row r="683" ht="14.25" customHeight="1" s="36"/>
-    <row r="684" ht="14.25" customHeight="1" s="36"/>
-    <row r="685" ht="14.25" customHeight="1" s="36"/>
-    <row r="686" ht="14.25" customHeight="1" s="36"/>
-    <row r="687" ht="14.25" customHeight="1" s="36"/>
-    <row r="688" ht="14.25" customHeight="1" s="36"/>
-    <row r="689" ht="14.25" customHeight="1" s="36"/>
-    <row r="690" ht="14.25" customHeight="1" s="36"/>
-    <row r="691" ht="14.25" customHeight="1" s="36"/>
-    <row r="692" ht="14.25" customHeight="1" s="36"/>
-    <row r="693" ht="14.25" customHeight="1" s="36"/>
-    <row r="694" ht="14.25" customHeight="1" s="36"/>
-    <row r="695" ht="14.25" customHeight="1" s="36"/>
-    <row r="696" ht="14.25" customHeight="1" s="36"/>
-    <row r="697" ht="14.25" customHeight="1" s="36"/>
-    <row r="698" ht="14.25" customHeight="1" s="36"/>
-    <row r="699" ht="14.25" customHeight="1" s="36"/>
-    <row r="700" ht="14.25" customHeight="1" s="36"/>
-    <row r="701" ht="14.25" customHeight="1" s="36"/>
-    <row r="702" ht="14.25" customHeight="1" s="36"/>
-    <row r="703" ht="14.25" customHeight="1" s="36"/>
-    <row r="704" ht="14.25" customHeight="1" s="36"/>
-    <row r="705" ht="14.25" customHeight="1" s="36"/>
-    <row r="706" ht="14.25" customHeight="1" s="36"/>
+    <row r="663" ht="14.25" customHeight="1" s="36">
+      <c r="A663" s="37" t="inlineStr">
+        <is>
+          <t>RH1</t>
+        </is>
+      </c>
+      <c r="B663" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C663" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D663" s="39" t="inlineStr">
+        <is>
+          <t>ปี 4 เทอม 1 กับเทอม 2 เทอมไหนต้องลงหน่วยกิตเยอะกว่ากัน</t>
+        </is>
+      </c>
+      <c r="E663" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F663" s="39" t="inlineStr">
+        <is>
+          <t>ภาค 1 12, ภาค 2 6</t>
+        </is>
+      </c>
+      <c r="G663" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 4 ภาคการศึกษาที่ 1 หนักกว่า (12 เทียบกับ 6 หน่วยกิต) ต่างกัน 6 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ AIT 2566 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 4 ภาคการศึกษาที่ 1: 12 หน่วยกิต (หน้า 26)
+- ปีที่ 4 ภาคการศึกษาที่ 2: 6 หน่วยกิต (หน้า 26)</t>
+        </is>
+      </c>
+      <c r="H663" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 26</t>
+        </is>
+      </c>
+      <c r="I663" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J663" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K663" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L663" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M663" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N663" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O663" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="664" ht="14.25" customHeight="1" s="36">
+      <c r="A664" s="37" t="inlineStr">
+        <is>
+          <t>RH2</t>
+        </is>
+      </c>
+      <c r="B664" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C664" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D664" s="39" t="inlineStr">
+        <is>
+          <t>ตามแผน ปี 4 ทั้งปีต้องเรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E664" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F664" s="39" t="inlineStr">
+        <is>
+          <t>12 + 6</t>
+        </is>
+      </c>
+      <c r="G664" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 4 ตามแผนปกติเรียนรวม 18 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ AIT 2566 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 4 ภาคการศึกษาที่ 1: 12 หน่วยกิต (หน้า 26)
+- ปีที่ 4 ภาคการศึกษาที่ 2: 6 หน่วยกิต (หน้า 26)</t>
+        </is>
+      </c>
+      <c r="H664" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 26</t>
+        </is>
+      </c>
+      <c r="I664" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J664" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K664" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L664" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M664" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N664" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O664" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="665" ht="14.25" customHeight="1" s="36">
+      <c r="A665" s="37" t="inlineStr">
+        <is>
+          <t>RH3</t>
+        </is>
+      </c>
+      <c r="B665" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C665" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D665" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าลงวิชาการเพิ่มประสิทธิภาพโครงข่ายประสาทเทียม และวิชาแคลคูลัส 1 รวมกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E665" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F665" s="39" t="inlineStr">
+        <is>
+          <t>3 + 3</t>
+        </is>
+      </c>
+      <c r="G665" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: รวม 6 หน่วยกิต (3 + 3)
+- 06046412 การเพิ่มประสิทธิภาพโครงข่ายประสาทเทียม (NEURAL NETWORK OPTIMIZATION) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 2
+- 06046400 แคลคูลัส 1 (CALCULUS 1) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H665" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 19, 20, 23, 24, 37, 38, 287, 295</t>
+        </is>
+      </c>
+      <c r="I665" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J665" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K665" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L665" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M665" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N665" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O665" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="666" ht="14.25" customHeight="1" s="36">
+      <c r="A666" s="37" t="inlineStr">
+        <is>
+          <t>RH4</t>
+        </is>
+      </c>
+      <c r="B666" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C666" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D666" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ทันลงวิชาการเรียนรู้ของเครื่องเชิงความน่าจะเป็น ตามแผน ไปลงตอนปี 3 แทนได้ไหม</t>
+        </is>
+      </c>
+      <c r="E666" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F666" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ตามแผนปี 2 ต้องผ่าน 06066001</t>
+        </is>
+      </c>
+      <c r="G666" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ได้ — ตามแผนวิชานี้อยู่ปีที่ 2 อยู่แล้ว (ต้องผ่านวิชาบังคับก่อนข้างต้นก่อน)
+วิชา 06046405 การเรียนรู้ของเครื่องเชิงความน่าจะเป็น (PROBABILISTIC MACHINE LEARNING) — 3(3-0-6) หน่วยกิต
+ตามแผนการศึกษา: ปีที่ 2 ภาคการศึกษาที่ 1
+วิชาบังคับก่อน (ต้องสอบผ่านก่อนจึงจะลงได้):
+  - 06066001 ความน่าจะเป็นและสถิติ (PROBABILITY AND STATISTICS) — ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H666" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 37, 291, 19, 20, 23, 24, 289</t>
+        </is>
+      </c>
+      <c r="I666" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (ปีตามแผน + วิชาบังคับก่อน → ลงได้/ไม่ได้) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J666" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="K666" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L666" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M666" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N666" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O666" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="667" ht="14.25" customHeight="1" s="36">
+      <c r="A667" s="37" t="inlineStr">
+        <is>
+          <t>RC1</t>
+        </is>
+      </c>
+      <c r="B667" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C667" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D667" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเรียนตามแผนครบถึงปี 2 แล้ว จะมีหน่วยกิตสะสมเท่าไร และเหลืออีกกี่หน่วยกิตถึงจะจบ</t>
+        </is>
+      </c>
+      <c r="E667" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F667" s="39" t="inlineStr">
+        <is>
+          <t>สะสม 71 เหลือ 49</t>
+        </is>
+      </c>
+      <c r="G667" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: เรียนครบตามแผนถึงปีที่ 2 มีหน่วยกิตสะสม 71 หน่วยกิต เหลืออีก 49 หน่วยกิตจึงครบ 120 หน่วยกิตตามเกณฑ์จบ (หน้า 5)
+หน่วยกิตต่อภาคตามแผนปกติของ AIT 2566 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 1 ภาคการศึกษาที่ 1: 15 หน่วยกิต (หน้า 23)
+- ปีที่ 1 ภาคการศึกษาที่ 2: 19 หน่วยกิต (หน้า 23)
+- ปีที่ 2 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 24)
+- ปีที่ 2 ภาคการศึกษาที่ 2: 19 หน่วยกิต (หน้า 24)</t>
+        </is>
+      </c>
+      <c r="H667" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 23, 24</t>
+        </is>
+      </c>
+      <c r="I667" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J667" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K667" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L667" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M667" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N667" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O667" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="668" ht="14.25" customHeight="1" s="36">
+      <c r="A668" s="37" t="inlineStr">
+        <is>
+          <t>RC2</t>
+        </is>
+      </c>
+      <c r="B668" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C668" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D668" s="39" t="inlineStr">
+        <is>
+          <t>กว่าจะได้ลงวิชาพื้นฐานการเรียนรู้เชิงลึก ต้องสอบผ่านกี่วิชา นับทุกทอด</t>
+        </is>
+      </c>
+      <c r="E668" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F668" s="39" t="inlineStr">
+        <is>
+          <t>3 วิชา: 06046400, 06046401, 06046402</t>
+        </is>
+      </c>
+      <c r="G668" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING) — ปีที่ 2 ภาคการศึกษาที่ 1
+วิชาที่ต้องสอบผ่านก่อน (↳ = วิชาที่ต้องผ่านก่อนวิชาด้านบนอีกชั้น):
+  • 06046401 แคลคูลัส 2 (CALCULUS 2) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2
+    ↳ 06046400 แคลคูลัส 1 (CALCULUS 1) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1
+  • 06046402 พีชคณิตเชิงเส้น (LINEAR ALGEBRA) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1
+รวมต้องผ่านก่อน 3 วิชา</t>
+        </is>
+      </c>
+      <c r="H668" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 37, 19, 292, 23, 287, 20, 24, 288</t>
+        </is>
+      </c>
+      <c r="I668" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (วิชาบังคับก่อนไล่หลายชั้น) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J668" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K668" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L668" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M668" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N668" s="39" t="inlineStr">
+        <is>
+          <t>0.02s</t>
+        </is>
+      </c>
+      <c r="O668" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="669" ht="14.25" customHeight="1" s="36">
+      <c r="A669" s="37" t="inlineStr">
+        <is>
+          <t>RH5</t>
+        </is>
+      </c>
+      <c r="B669" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C669" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D669" s="39" t="inlineStr">
+        <is>
+          <t>ปี 3 เทอม 1 กับเทอม 2 เทอมไหนต้องลงหน่วยกิตเยอะกว่ากัน</t>
+        </is>
+      </c>
+      <c r="E669" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F669" s="39" t="inlineStr">
+        <is>
+          <t>ภาค 1 18, ภาค 2 9</t>
+        </is>
+      </c>
+      <c r="G669" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 3 ภาคการศึกษาที่ 1 หนักกว่า (18 เทียบกับ 12 หน่วยกิต) ต่างกัน 6 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ BIT 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 3 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 28)
+- ปีที่ 3 ภาคการศึกษาที่ 2: 12 หน่วยกิต (หน้า 29)</t>
+        </is>
+      </c>
+      <c r="H669" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 28, 29</t>
+        </is>
+      </c>
+      <c r="I669" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J669" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K669" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L669" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M669" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N669" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O669" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="670" ht="14.25" customHeight="1" s="36">
+      <c r="A670" s="37" t="inlineStr">
+        <is>
+          <t>RH6</t>
+        </is>
+      </c>
+      <c r="B670" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C670" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D670" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าลงวิชาโครงงานทางด้านเทคโนโลยีสารสนเทศเชิงธุรกิจ 2 และวิชาการแก้ปัญหาทางด้านเทคโนโลยีสารสนเทศ รวมกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E670" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F670" s="39" t="inlineStr">
+        <is>
+          <t>3 + 3</t>
+        </is>
+      </c>
+      <c r="G670" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: รวม 6 หน่วยกิต (3 + 3)
+- 06036146 โครงงานทางด้านเทคโนโลยีสารสนเทศเชิงธุรกิจ 2 (PROJECT IN BUSINESS INFORMATION TECHNOLOGY 2) — 3(0-9-0) | ปีที่ 4 ภาคการศึกษาที่ 1
+- 06036118 การแก้ปัญหาทางด้านเทคโนโลยีสารสนเทศ (PROBLEM SOLVING IN INFORMATION TECHNOLOGY) — 3(2-2-5) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H670" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 23, 26, 29, 31, 75, 76, 246, 256</t>
+        </is>
+      </c>
+      <c r="I670" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J670" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K670" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L670" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M670" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N670" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O670" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="671" ht="14.25" customHeight="1" s="36">
+      <c r="A671" s="37" t="inlineStr">
+        <is>
+          <t>RH7</t>
+        </is>
+      </c>
+      <c r="B671" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C671" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D671" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ทันลงวิชาการพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก ตามแผน ไปลงตอนปี 4 แทนได้ไหม</t>
+        </is>
+      </c>
+      <c r="E671" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F671" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ตามแผนปี 3 ต้องผ่าน 06036119</t>
+        </is>
+      </c>
+      <c r="G671" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ได้ — ตามแผนวิชานี้อยู่ปีที่ 3 อยู่แล้ว (ต้องผ่านวิชาบังคับก่อนข้างต้นก่อน)
+วิชา 06036114 การพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก (WEB APPLICATION DEVELOPMENT USING FRAMEWORKS) — 3(2-2-5) หน่วยกิต
+ตามแผนการศึกษา: ปีที่ 3 ภาคการศึกษาที่ 1
+วิชาบังคับก่อน (ต้องสอบผ่านก่อนจึงจะลงได้):
+  - 06036119 พื้นฐานการเขียนโปรแกรม (PROGRAMMING FUNDAMENTALS) — ปีที่ 1 ภาคการศึกษาที่ 2
+  - 06036122 การสื่อสารด้วยภาพสำหรับธุรกิจ (VISUAL COMMUNICATION FOR BUSINESS) — ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H671" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 75, 23, 244, 270, 22, 27, 28, 32</t>
+        </is>
+      </c>
+      <c r="I671" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (ปีตามแผน + วิชาบังคับก่อน → ลงได้/ไม่ได้) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J671" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K671" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L671" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M671" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N671" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O671" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="672" ht="14.25" customHeight="1" s="36">
+      <c r="A672" s="37" t="inlineStr">
+        <is>
+          <t>RC3</t>
+        </is>
+      </c>
+      <c r="B672" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C672" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D672" s="39" t="inlineStr">
+        <is>
+          <t>กว่าจะได้ลงวิชาการพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก ต้องสอบผ่านกี่วิชา นับทุกทอด</t>
+        </is>
+      </c>
+      <c r="E672" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F672" s="39" t="inlineStr">
+        <is>
+          <t>2 วิชา: 06036119, 06036122</t>
+        </is>
+      </c>
+      <c r="G672" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06036114 การพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก (WEB APPLICATION DEVELOPMENT USING FRAMEWORKS) — ปีที่ 3 ภาคการศึกษาที่ 1
+วิชาที่ต้องสอบผ่านก่อน (↳ = วิชาที่ต้องผ่านก่อนวิชาด้านบนอีกชั้น):
+  • 06036119 พื้นฐานการเขียนโปรแกรม (PROGRAMMING FUNDAMENTALS) — 3(2-2-5) | ปีที่ 1 ภาคการศึกษาที่ 2
+  • 06036122 การสื่อสารด้วยภาพสำหรับธุรกิจ (VISUAL COMMUNICATION FOR BUSINESS) — 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 1
+รวมต้องผ่านก่อน 2 วิชา</t>
+        </is>
+      </c>
+      <c r="H672" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 75, 23, 244, 270, 22, 27, 28, 32</t>
+        </is>
+      </c>
+      <c r="I672" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (วิชาบังคับก่อนไล่หลายชั้น) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J672" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K672" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L672" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M672" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N672" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O672" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="673" ht="14.25" customHeight="1" s="36">
+      <c r="A673" s="37" t="inlineStr">
+        <is>
+          <t>RH8</t>
+        </is>
+      </c>
+      <c r="B673" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C673" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D673" s="39" t="inlineStr">
+        <is>
+          <t>ปี 1 เทอม 1 กับเทอม 2 เทอมไหนต้องลงหน่วยกิตเยอะกว่ากัน</t>
+        </is>
+      </c>
+      <c r="E673" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F673" s="39" t="inlineStr">
+        <is>
+          <t>ภาค 1 18, ภาค 2 21</t>
+        </is>
+      </c>
+      <c r="G673" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 1 ภาคการศึกษาที่ 2 หนักกว่า (21 เทียบกับ 18 หน่วยกิต) ต่างกัน 3 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ DSBA 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 1 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 23)
+- ปีที่ 1 ภาคการศึกษาที่ 2: 21 หน่วยกิต (หน้า 24)</t>
+        </is>
+      </c>
+      <c r="H673" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 23, 24</t>
+        </is>
+      </c>
+      <c r="I673" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J673" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K673" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L673" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M673" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N673" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O673" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="674" ht="14.25" customHeight="1" s="36">
+      <c r="A674" s="37" t="inlineStr">
+        <is>
+          <t>RH9</t>
+        </is>
+      </c>
+      <c r="B674" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C674" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D674" s="39" t="inlineStr">
+        <is>
+          <t>ตามแผน ปี 3 ทั้งปีต้องเรียนกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E674" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F674" s="39" t="inlineStr">
+        <is>
+          <t>18 + 18</t>
+        </is>
+      </c>
+      <c r="G674" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 3 ตามแผนปกติเรียนรวม 36 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ DSBA 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 3 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 27)
+- ปีที่ 3 ภาคการศึกษาที่ 2: 18 หน่วยกิต (หน้า 28)</t>
+        </is>
+      </c>
+      <c r="H674" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 27, 28</t>
+        </is>
+      </c>
+      <c r="I674" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J674" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K674" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L674" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M674" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N674" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O674" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="675" ht="14.25" customHeight="1" s="36">
+      <c r="A675" s="37" t="inlineStr">
+        <is>
+          <t>RH10</t>
+        </is>
+      </c>
+      <c r="B675" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C675" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D675" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าลงวิชาการเรียนรู้ของเครื่องเชิงประยุกต์ และวิชาการสื่อสารและการนำเสนออย่างมืออาชีพ รวมกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E675" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F675" s="39" t="inlineStr">
+        <is>
+          <t>3 + 3</t>
+        </is>
+      </c>
+      <c r="G675" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: รวม 6 หน่วยกิต (3 + 3)
+- 06026211 การเรียนรู้ของเครื่องเชิงประยุกต์ (APPLIED MACHINE LEARNING) — 3(2-2-5) | ปีที่ 3 ภาคการศึกษาที่ 1
+- 90644042 การสื่อสารและการนำเสนออย่างมืออาชีพ (PROFESSIONAL COMMUNICATION AND PRESENTATION) — 3(3-0-6) | ปีที่ 3 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H675" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 27, 34, 16, 18, 68, 323, 353, 354</t>
+        </is>
+      </c>
+      <c r="I675" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J675" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K675" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L675" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M675" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N675" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O675" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="676" ht="14.25" customHeight="1" s="36">
+      <c r="A676" s="37" t="inlineStr">
+        <is>
+          <t>RH11</t>
+        </is>
+      </c>
+      <c r="B676" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C676" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D676" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ทันลงวิชาระบบสารสนเทศเพื่อการจัดการ ตามแผน ไปลงตอนปี 3 แทนได้ไหม</t>
+        </is>
+      </c>
+      <c r="E676" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F676" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ตามแผนปี 2 ต้องผ่าน 06066101</t>
+        </is>
+      </c>
+      <c r="G676" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ได้ — ตามแผนวิชานี้อยู่ปีที่ 2 อยู่แล้ว (ต้องผ่านวิชาบังคับก่อนข้างต้นก่อน)
+วิชา 06066102 ระบบสารสนเทศเพื่อการจัดการ (MANAGEMENT INFORMATION SYSTEMS) — 3(3-0-6) หน่วยกิต
+ตามแผนการศึกษา: ปีที่ 2 ภาคการศึกษาที่ 2
+วิชาบังคับก่อน (ต้องสอบผ่านก่อนจึงจะลงได้):
+  - 06066101 พื้นฐานทางธุรกิจสำหรับเทคโนโลยีสารสนเทศ (BUSINESS FUNDAMENTALS FOR INFORMATION TECHNOLOGY) — ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H676" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 18, 73, 353, 23, 26, 30, 33, 317</t>
+        </is>
+      </c>
+      <c r="I676" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (ปีตามแผน + วิชาบังคับก่อน → ลงได้/ไม่ได้) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J676" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K676" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L676" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M676" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N676" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O676" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="677" ht="14.25" customHeight="1" s="36">
+      <c r="A677" s="37" t="inlineStr">
+        <is>
+          <t>RC4</t>
+        </is>
+      </c>
+      <c r="B677" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C677" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D677" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเรียนตามแผนครบถึงปี 3 แล้ว จะมีหน่วยกิตสะสมเท่าไร และเหลืออีกกี่หน่วยกิตถึงจะจบ</t>
+        </is>
+      </c>
+      <c r="E677" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F677" s="39" t="inlineStr">
+        <is>
+          <t>สะสม 114 เหลือ 18</t>
+        </is>
+      </c>
+      <c r="G677" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: เรียนครบตามแผนถึงปีที่ 3 มีหน่วยกิตสะสม 114 หน่วยกิต เหลืออีก 18 หน่วยกิตจึงครบ 132 หน่วยกิตตามเกณฑ์จบ (หน้า 2)
+หน่วยกิตต่อภาคตามแผนปกติของ DSBA 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 1 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 23)
+- ปีที่ 1 ภาคการศึกษาที่ 2: 21 หน่วยกิต (หน้า 24)
+- ปีที่ 2 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 25)
+- ปีที่ 2 ภาคการศึกษาที่ 2: 21 หน่วยกิต (หน้า 26)
+- ปีที่ 3 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 27)
+- ปีที่ 3 ภาคการศึกษาที่ 2: 18 หน่วยกิต (หน้า 28)</t>
+        </is>
+      </c>
+      <c r="H677" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 23, 24, 25, 26, 27, 28</t>
+        </is>
+      </c>
+      <c r="I677" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J677" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="K677" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L677" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M677" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N677" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O677" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="678" ht="14.25" customHeight="1" s="36">
+      <c r="A678" s="37" t="inlineStr">
+        <is>
+          <t>RH12</t>
+        </is>
+      </c>
+      <c r="B678" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C678" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D678" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าลงวิชาระบบโครงสร้างพื้นฐานและการบริการ และวิชาการวิเคราะห์และออกแบบระบบสารสนเทศ รวมกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E678" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F678" s="39" t="inlineStr">
+        <is>
+          <t>3 + 3</t>
+        </is>
+      </c>
+      <c r="G678" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: รวม 6 หน่วยกิต (3 + 3)
+- 06016420 ระบบโครงสร้างพื้นฐานและการบริการ (INFRASTRUCTURE SYSTEMS AND SERVICES) — 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 2
+- 06066304 การวิเคราะห์และออกแบบระบบสารสนเทศ (INFORMATION SYSTEM ANALYSIS AND DESIGN) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H678" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 24, 25, 33, 34, 84, 88, 332, 337</t>
+        </is>
+      </c>
+      <c r="I678" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J678" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K678" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L678" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M678" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N678" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O678" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="679" ht="14.25" customHeight="1" s="36">
+      <c r="A679" s="37" t="inlineStr">
+        <is>
+          <t>RH13</t>
+        </is>
+      </c>
+      <c r="B679" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C679" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D679" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ทันลงวิชาโครงสร้างพื้นฐานเครือข่ายการสื่อสาร ตามแผน ไปลงตอนปี 3 แทนได้ไหม</t>
+        </is>
+      </c>
+      <c r="E679" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F679" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ตามแผนปี 2 ต้องผ่าน 06016413</t>
+        </is>
+      </c>
+      <c r="G679" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ได้ — ตามแผนวิชานี้อยู่ปีที่ 2 อยู่แล้ว (ต้องผ่านวิชาบังคับก่อนข้างต้นก่อน)
+วิชา 06016419 โครงสร้างพื้นฐานเครือข่ายการสื่อสาร (COMMUNICATION NETWORK INFRASTRUCTURE) — 3(2-2-5) หน่วยกิต
+ตามแผนการศึกษา: ปีที่ 2 ภาคการศึกษาที่ 2
+วิชาบังคับก่อน (ต้องสอบผ่านก่อนจึงจะลงได้):
+  - 06016413 ระบบเครือข่ายเบื้องต้น (INTRODUCTION TO NETWORK SYSTEMS) — ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H679" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 84, 24, 25, 33, 34, 40, 328, 331</t>
+        </is>
+      </c>
+      <c r="I679" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (ปีตามแผน + วิชาบังคับก่อน → ลงได้/ไม่ได้) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J679" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K679" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L679" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M679" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N679" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O679" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="680" ht="14.25" customHeight="1" s="36">
+      <c r="A680" s="37" t="inlineStr">
+        <is>
+          <t>RC5</t>
+        </is>
+      </c>
+      <c r="B680" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C680" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D680" s="39" t="inlineStr">
+        <is>
+          <t>จบมาด้วยเกรดเฉลี่ย 3.74 ได้เหรียญทองไหม</t>
+        </is>
+      </c>
+      <c r="E680" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F680" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ได้ (ต้อง &gt;= 3.75) ได้อันดับ 1</t>
+        </is>
+      </c>
+      <c r="G680" s="39" t="inlineStr">
+        <is>
+          <t>ปริญญาเกียรตินิยม — ข้อ 36 ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 88, 89
+(ข้อบังคับของสถาบัน ใช้กับทุกหลักสูตรปริญญาตรี)
+- เกียรตินิยมอันดับหนึ่งและเหรียญทอง: ค่าระดับคะแนนเฉลี่ยสะสมตามโครงสร้างหลักสูตรสูงสุดในกลุ่มผู้สำเร็จการศึกษาปีเดียวกันของหลักสูตร และค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.75 และต้องไม่เทียบโอนผลการเรียนจากสถาบันอื่น
+- เกียรตินิยมอันดับหนึ่ง: ค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.50
+- เกียรตินิยมอันดับสอง: ค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.25
+- กรณีโอนผลการเรียนจากสถาบันอื่น ทุกรายวิชาต้องได้ไม่ต่ำกว่า B หรือ S และต้องเรียนในหลักสูตรของสถาบันไม่น้อยกว่า 2 ใน 3 ของหน่วยกิตรวม
+- เงื่อนไขทั่วไป (ข้อ 36.1): เรียนไม่เกินระยะเวลาตามแผนการศึกษา · ไม่มีรายวิชาใดได้ F หรือ U · ไม่เคยเรียนซ้ำเพื่อเปลี่ยนเกรด · ไม่เคยลาพักเพราะไม่ลงทะเบียนตามกำหนด และไม่เคยถูกลงโทษทางวินัย</t>
+        </is>
+      </c>
+      <c r="H680" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 88, 89</t>
+        </is>
+      </c>
+      <c r="I680" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J680" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K680" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L680" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M680" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N680" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O680" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="681" ht="14.25" customHeight="1" s="36">
+      <c r="A681" s="37" t="inlineStr">
+        <is>
+          <t>RC6</t>
+        </is>
+      </c>
+      <c r="B681" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C681" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D681" s="39" t="inlineStr">
+        <is>
+          <t>ปีสี่เทอมสุดท้ายเหลือ 24 หน่วยกิต ลงทีเดียวหมดได้ไหม</t>
+        </is>
+      </c>
+      <c r="E681" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F681" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ข้อยกเว้นปีสุดท้ายไม่เกิน 27</t>
+        </is>
+      </c>
+      <c r="G681" s="39" t="inlineStr">
+        <is>
+          <t>ได้ — นักศึกษาชั้นปีสุดท้ายที่เหลือหน่วยกิตน้อยกว่า 9 หน่วยกิตหรือต้องลงเกิน 22 หน่วยกิตเพื่อสำเร็จการศึกษา สามารถลงทะเบียนได้ไม่เกิน 27 หน่วยกิตตามข้อยกเว้นในข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวก มคอ.2 AIT 2566) หน้า 82 ซึ่งครอบคลุมกรณีนี้ โดยหลักสูตรวท.บ. (เทคโนโลยีสารสนเทศ) ต้องเรียนรวม 129 หน่วยกิต (ข้อมูลจาก มคอ.2 หลักสูตร IT 2565 หน้า 6)</t>
+        </is>
+      </c>
+      <c r="H681" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 82</t>
+        </is>
+      </c>
+      <c r="I681" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) → Typhoon เรียบเรียง</t>
+        </is>
+      </c>
+      <c r="J681" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K681" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L681" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M681" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก ข้อบังคับ ป.ตรี (AIT 2566 ภาคผนวก หน้า 82, 87, 89))</t>
+        </is>
+      </c>
+      <c r="N681" s="39" t="inlineStr">
+        <is>
+          <t>2.13s</t>
+        </is>
+      </c>
+      <c r="O681" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="682" ht="14.25" customHeight="1" s="36">
+      <c r="A682" s="37" t="inlineStr">
+        <is>
+          <t>RC7</t>
+        </is>
+      </c>
+      <c r="B682" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C682" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D682" s="39" t="inlineStr">
+        <is>
+          <t>โดนภาคทัณฑ์แล้วต้องทำยังไงถึงจะพ้น</t>
+        </is>
+      </c>
+      <c r="E682" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F682" s="39" t="inlineStr">
+        <is>
+          <t>เกรดเฉลี่ยสะสมไม่ต่ำกว่า 2.00</t>
+        </is>
+      </c>
+      <c r="G682" s="39" t="inlineStr">
+        <is>
+          <t>การภาคทัณฑ์ — ข้อ 31 ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 87
+(ข้อบังคับของสถาบัน ใช้กับทุกหลักสูตรปริญญาตรี)
+- นักศึกษาที่ได้ค่าระดับคะแนนเฉลี่ยสะสมต่ำกว่า 2.00 ต้องถูกภาคทัณฑ์
+- จะพ้นภาคทัณฑ์เมื่อค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 2.00 (นับรวมภาคการศึกษาพิเศษด้วย)
+- ถ้าระหว่างภาคทัณฑ์ได้ค่าระดับคะแนนเฉลี่ยประจำภาคถัดไปต่ำกว่า 2.00 จะพ้นสภาพนักศึกษา (ข้อ 43.10)</t>
+        </is>
+      </c>
+      <c r="H682" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 87</t>
+        </is>
+      </c>
+      <c r="I682" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J682" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K682" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L682" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M682" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก ข้อบังคับ ป.ตรี (AIT 2566 ภาคผนวก หน้า 82, 87, 89))</t>
+        </is>
+      </c>
+      <c r="N682" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O682" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="683" ht="14.25" customHeight="1" s="36">
+      <c r="A683" s="37" t="inlineStr">
+        <is>
+          <t>RC8</t>
+        </is>
+      </c>
+      <c r="B683" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C683" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D683" s="39" t="inlineStr">
+        <is>
+          <t>สะสมได้ 117 หน่วยกิต GPA 3.20 ขาดอีกกี่หน่วยกิตถึงจบ</t>
+        </is>
+      </c>
+      <c r="E683" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F683" s="39" t="inlineStr">
+        <is>
+          <t>ขาด 3</t>
+        </is>
+      </c>
+      <c r="G683" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ยังจบไม่ได้
+หลักสูตร AIT 2566 (ปริญญาตรี) ต้องเรียนครบไม่น้อยกว่า 120 หน่วยกิต (หน้า 5)
+- หน่วยกิต: เก็บได้ 117 หน่วยกิต → ยังขาดอีก 3 หน่วยกิต (ต้องครบ 120)
+- เกรดเฉลี่ยสะสม 3.20 → ผ่านเกณฑ์ขั้นต่ำ 2.00 (ข้อ 34)
+- เงื่อนไขอื่นตามข้อ 34: สอบผ่านทุกรายวิชาตามโครงสร้างหลักสูตร และผ่านการสอบภาษาอังกฤษ (English Exit exam)</t>
+        </is>
+      </c>
+      <c r="H683" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 5, 88</t>
+        </is>
+      </c>
+      <c r="I683" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวม + เกรดขั้นต่ำ ข้อ 34) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J683" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K683" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L683" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M683" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N683" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O683" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="684" ht="14.25" customHeight="1" s="36">
+      <c r="A684" s="37" t="inlineStr">
+        <is>
+          <t>RC9</t>
+        </is>
+      </c>
+      <c r="B684" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C684" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D684" s="39" t="inlineStr">
+        <is>
+          <t>BIT กับ DSBA ต้องเรียนรวมต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E684" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 8 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F684" s="39" t="inlineStr">
+        <is>
+          <t>ต่างกัน 6</t>
+        </is>
+      </c>
+      <c r="G684" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ต่างกัน 6 หน่วยกิต (DSBA 2565 (ปริญญาตรี) มากกว่า BIT 2565 (ปริญญาตรี))
+- BIT 2565 (ปริญญาตรี): ไม่น้อยกว่า 126 หน่วยกิต (หน้า 6)
+- DSBA 2565 (ปริญญาตรี): ไม่น้อยกว่า 132 หน่วยกิต (หน้า 2)</t>
+        </is>
+      </c>
+      <c r="H684" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 6, 2</t>
+        </is>
+      </c>
+      <c r="I684" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมข้ามหลักสูตร) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J684" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K684" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L684" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M684" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N684" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O684" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="685" ht="14.25" customHeight="1" s="36">
+      <c r="A685" s="37" t="inlineStr">
+        <is>
+          <t>SH1</t>
+        </is>
+      </c>
+      <c r="B685" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C685" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D685" s="39" t="inlineStr">
+        <is>
+          <t>ปี 2 ภาคต้นกับภาคปลาย ภาคไหนเรียนหนักกว่า ต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E685" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F685" s="39" t="inlineStr">
+        <is>
+          <t>ภาค 1 18, ภาค 2 19</t>
+        </is>
+      </c>
+      <c r="G685" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 2 ภาคการศึกษาที่ 2 หนักกว่า (19 เทียบกับ 18 หน่วยกิต) ต่างกัน 1 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ AIT 2566 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 2 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 24)
+- ปีที่ 2 ภาคการศึกษาที่ 2: 19 หน่วยกิต (หน้า 24)</t>
+        </is>
+      </c>
+      <c r="H685" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 24</t>
+        </is>
+      </c>
+      <c r="I685" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J685" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K685" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L685" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M685" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N685" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O685" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="686" ht="14.25" customHeight="1" s="36">
+      <c r="A686" s="37" t="inlineStr">
+        <is>
+          <t>SH2</t>
+        </is>
+      </c>
+      <c r="B686" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C686" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D686" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเรียนตามแผน ตลอดปีที่ 2 รวมสองเทอมได้กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E686" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F686" s="39" t="inlineStr">
+        <is>
+          <t>18 + 19</t>
+        </is>
+      </c>
+      <c r="G686" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 2 ตามแผนปกติเรียนรวม 37 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ AIT 2566 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 2 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 24)
+- ปีที่ 2 ภาคการศึกษาที่ 2: 19 หน่วยกิต (หน้า 24)</t>
+        </is>
+      </c>
+      <c r="H686" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 24</t>
+        </is>
+      </c>
+      <c r="I686" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J686" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K686" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L686" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M686" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N686" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O686" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="687" ht="14.25" customHeight="1" s="36">
+      <c r="A687" s="37" t="inlineStr">
+        <is>
+          <t>SH3</t>
+        </is>
+      </c>
+      <c r="B687" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C687" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D687" s="39" t="inlineStr">
+        <is>
+          <t>วิชาสัมมนาปัญญาประดิษฐ์ บวก พลเมืองดิจิทัล ได้หน่วยกิตรวมเท่าไร</t>
+        </is>
+      </c>
+      <c r="E687" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F687" s="39" t="inlineStr">
+        <is>
+          <t>3 + 3</t>
+        </is>
+      </c>
+      <c r="G687" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: รวม 6 หน่วยกิต (3 + 3)
+- 06046440 วิชาสัมมนาปัญญาประดิษฐ์ (SEMINAR IN ARTIFICIAL INTELLIGENCE) — 3(2-2-5) | ปีที่ 3 ภาคการศึกษาที่ 1
+- 90641007 พลเมืองดิจิทัล (DIGITAL CITIZEN) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2</t>
+        </is>
+      </c>
+      <c r="H687" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 19, 22, 23, 25, 36, 40, 119, 120</t>
+        </is>
+      </c>
+      <c r="I687" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J687" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K687" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L687" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M687" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N687" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O687" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="688" ht="14.25" customHeight="1" s="36">
+      <c r="A688" s="37" t="inlineStr">
+        <is>
+          <t>SH4</t>
+        </is>
+      </c>
+      <c r="B688" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C688" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D688" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเลื่อนวิชาแคลคูลัส 2 ไปเรียนปี 2 จะได้หรือเปล่า</t>
+        </is>
+      </c>
+      <c r="E688" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F688" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ตามแผนปี 1 ต้องผ่าน 06046400</t>
+        </is>
+      </c>
+      <c r="G688" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ได้ — ตามแผนวิชานี้อยู่ปีที่ 1 อยู่แล้ว (ต้องผ่านวิชาบังคับก่อนข้างต้นก่อน)
+วิชา 06046401 แคลคูลัส 2 (CALCULUS 2) — 3(3-0-6) หน่วยกิต
+ตามแผนการศึกษา: ปีที่ 1 ภาคการศึกษาที่ 2
+วิชาบังคับก่อน (ต้องสอบผ่านก่อนจึงจะลงได้):
+  - 06046400 แคลคูลัส 1 (CALCULUS 1) — ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H688" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 19, 37, 287, 23, 292</t>
+        </is>
+      </c>
+      <c r="I688" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (ปีตามแผน + วิชาบังคับก่อน → ลงได้/ไม่ได้) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J688" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="K688" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L688" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M688" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N688" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O688" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="689" ht="14.25" customHeight="1" s="36">
+      <c r="A689" s="37" t="inlineStr">
+        <is>
+          <t>SC1</t>
+        </is>
+      </c>
+      <c r="B689" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C689" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D689" s="39" t="inlineStr">
+        <is>
+          <t>จบปี 3 ตามแผนพอดี เก็บหน่วยกิตได้กี่หน่วยกิต ยังขาดอีกเท่าไหร่</t>
+        </is>
+      </c>
+      <c r="E689" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F689" s="39" t="inlineStr">
+        <is>
+          <t>สะสม 102 เหลือ 18</t>
+        </is>
+      </c>
+      <c r="G689" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: เรียนครบตามแผนถึงปีที่ 3 มีหน่วยกิตสะสม 102 หน่วยกิต เหลืออีก 18 หน่วยกิตจึงครบ 120 หน่วยกิตตามเกณฑ์จบ (หน้า 5)
+หน่วยกิตต่อภาคตามแผนปกติของ AIT 2566 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 1 ภาคการศึกษาที่ 1: 15 หน่วยกิต (หน้า 23)
+- ปีที่ 1 ภาคการศึกษาที่ 2: 19 หน่วยกิต (หน้า 23)
+- ปีที่ 2 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 24)
+- ปีที่ 2 ภาคการศึกษาที่ 2: 19 หน่วยกิต (หน้า 24)
+- ปีที่ 3 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 25)
+- ปีที่ 3 ภาคการศึกษาที่ 2: 13 หน่วยกิต (หน้า 25)</t>
+        </is>
+      </c>
+      <c r="H689" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 23, 24, 25</t>
+        </is>
+      </c>
+      <c r="I689" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J689" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="K689" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L689" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M689" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N689" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O689" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="690" ht="14.25" customHeight="1" s="36">
+      <c r="A690" s="37" t="inlineStr">
+        <is>
+          <t>SC2</t>
+        </is>
+      </c>
+      <c r="B690" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C690" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D690" s="39" t="inlineStr">
+        <is>
+          <t>วิชาพื้นฐานการเรียนรู้เชิงลึก มีวิชาที่ต้องผ่านก่อนทั้งทางตรงและทางอ้อมกี่วิชา อะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="E690" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F690" s="39" t="inlineStr">
+        <is>
+          <t>3 วิชา: 06046400, 06046401, 06046402</t>
+        </is>
+      </c>
+      <c r="G690" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06046406 พื้นฐานการเรียนรู้เชิงลึก (FUNDAMENTALS OF DEEP LEARNING) — ปีที่ 2 ภาคการศึกษาที่ 1
+วิชาที่ต้องสอบผ่านก่อน (↳ = วิชาที่ต้องผ่านก่อนวิชาด้านบนอีกชั้น):
+  • 06046401 แคลคูลัส 2 (CALCULUS 2) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2
+    ↳ 06046400 แคลคูลัส 1 (CALCULUS 1) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1
+  • 06046402 พีชคณิตเชิงเส้น (LINEAR ALGEBRA) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1
+รวมต้องผ่านก่อน 3 วิชา</t>
+        </is>
+      </c>
+      <c r="H690" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 37, 19, 292, 23, 287, 20, 24, 288</t>
+        </is>
+      </c>
+      <c r="I690" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (วิชาบังคับก่อนไล่หลายชั้น) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J690" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K690" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L690" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M690" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/AIT/AIT_academic_plan.json)</t>
+        </is>
+      </c>
+      <c r="N690" s="39" t="inlineStr">
+        <is>
+          <t>0.02s</t>
+        </is>
+      </c>
+      <c r="O690" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="691" ht="14.25" customHeight="1" s="36">
+      <c r="A691" s="37" t="inlineStr">
+        <is>
+          <t>SH5</t>
+        </is>
+      </c>
+      <c r="B691" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C691" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D691" s="39" t="inlineStr">
+        <is>
+          <t>ปี 3 ภาคต้นกับภาคปลาย ภาคไหนเรียนหนักกว่า ต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E691" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F691" s="39" t="inlineStr">
+        <is>
+          <t>ภาค 1 18, ภาค 2 9</t>
+        </is>
+      </c>
+      <c r="G691" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 3 ภาคการศึกษาที่ 1 หนักกว่า (18 เทียบกับ 12 หน่วยกิต) ต่างกัน 6 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ BIT 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 3 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 28)
+- ปีที่ 3 ภาคการศึกษาที่ 2: 12 หน่วยกิต (หน้า 29)</t>
+        </is>
+      </c>
+      <c r="H691" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 28, 29</t>
+        </is>
+      </c>
+      <c r="I691" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J691" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K691" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L691" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M691" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N691" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O691" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="692" ht="14.25" customHeight="1" s="36">
+      <c r="A692" s="37" t="inlineStr">
+        <is>
+          <t>SH6</t>
+        </is>
+      </c>
+      <c r="B692" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C692" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D692" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเรียนตามแผน ตลอดปีที่ 4 รวมสองเทอมได้กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E692" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F692" s="39" t="inlineStr">
+        <is>
+          <t>12 + 12</t>
+        </is>
+      </c>
+      <c r="G692" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 4 ตามแผนปกติเรียนรวม 24 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ BIT 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 4 ภาคการศึกษาที่ 1: 12 หน่วยกิต (หน้า 29)
+- ปีที่ 4 ภาคการศึกษาที่ 2: 12 หน่วยกิต (หน้า 30)</t>
+        </is>
+      </c>
+      <c r="H692" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 29, 30</t>
+        </is>
+      </c>
+      <c r="I692" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J692" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K692" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L692" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M692" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N692" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O692" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="693" ht="14.25" customHeight="1" s="36">
+      <c r="A693" s="37" t="inlineStr">
+        <is>
+          <t>SH7</t>
+        </is>
+      </c>
+      <c r="B693" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C693" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D693" s="39" t="inlineStr">
+        <is>
+          <t>ภาษาอังกฤษพื้นฐาน 2 บวก คณิตศาสตร์สำหรับธุรกิจ ได้หน่วยกิตรวมเท่าไร</t>
+        </is>
+      </c>
+      <c r="E693" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F693" s="39" t="inlineStr">
+        <is>
+          <t>3 + 3</t>
+        </is>
+      </c>
+      <c r="G693" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: รวม 6 หน่วยกิต (3 + 3)
+- 96644008 ภาษาอังกฤษพื้นฐาน 2 (FOUNDATION ENGLISH 2) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 2
+- 06036101 คณิตศาสตร์สำหรับธุรกิจ (MATHEMATICS FOR BUSINESS) — 3(3-0-6) | ปีที่ 1 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H693" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 20, 21, 26, 27, 31, 32, 74, 238</t>
+        </is>
+      </c>
+      <c r="I693" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J693" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K693" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L693" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M693" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N693" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O693" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="694" ht="14.25" customHeight="1" s="36">
+      <c r="A694" s="37" t="inlineStr">
+        <is>
+          <t>SH8</t>
+        </is>
+      </c>
+      <c r="B694" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C694" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D694" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเลื่อนวิชาการพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก ไปเรียนปี 4 จะได้หรือเปล่า</t>
+        </is>
+      </c>
+      <c r="E694" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F694" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ตามแผนปี 3 ต้องผ่าน 06036119</t>
+        </is>
+      </c>
+      <c r="G694" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ได้ — ตามแผนวิชานี้อยู่ปีที่ 3 อยู่แล้ว (ต้องผ่านวิชาบังคับก่อนข้างต้นก่อน)
+วิชา 06036114 การพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก (WEB APPLICATION DEVELOPMENT USING FRAMEWORKS) — 3(2-2-5) หน่วยกิต
+ตามแผนการศึกษา: ปีที่ 3 ภาคการศึกษาที่ 1
+วิชาบังคับก่อน (ต้องสอบผ่านก่อนจึงจะลงได้):
+  - 06036119 พื้นฐานการเขียนโปรแกรม (PROGRAMMING FUNDAMENTALS) — ปีที่ 1 ภาคการศึกษาที่ 2
+  - 06036122 การสื่อสารด้วยภาพสำหรับธุรกิจ (VISUAL COMMUNICATION FOR BUSINESS) — ปีที่ 2 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H694" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 75, 23, 244, 270, 22, 27, 28, 32</t>
+        </is>
+      </c>
+      <c r="I694" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (ปีตามแผน + วิชาบังคับก่อน → ลงได้/ไม่ได้) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J694" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K694" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L694" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M694" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N694" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O694" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="695" ht="14.25" customHeight="1" s="36">
+      <c r="A695" s="37" t="inlineStr">
+        <is>
+          <t>SC3</t>
+        </is>
+      </c>
+      <c r="B695" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C695" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D695" s="39" t="inlineStr">
+        <is>
+          <t>วิชาการพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก มีวิชาที่ต้องผ่านก่อนทั้งทางตรงและทางอ้อมกี่วิชา อะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="E695" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F695" s="39" t="inlineStr">
+        <is>
+          <t>2 วิชา: 06036119, 06036122</t>
+        </is>
+      </c>
+      <c r="G695" s="39" t="inlineStr">
+        <is>
+          <t>วิชา 06036114 การพัฒนาเว็บแอปพลิเคชันโดยใช้เฟรมเวิร์ก (WEB APPLICATION DEVELOPMENT USING FRAMEWORKS) — ปีที่ 3 ภาคการศึกษาที่ 1
+วิชาที่ต้องสอบผ่านก่อน (↳ = วิชาที่ต้องผ่านก่อนวิชาด้านบนอีกชั้น):
+  • 06036119 พื้นฐานการเขียนโปรแกรม (PROGRAMMING FUNDAMENTALS) — 3(2-2-5) | ปีที่ 1 ภาคการศึกษาที่ 2
+  • 06036122 การสื่อสารด้วยภาพสำหรับธุรกิจ (VISUAL COMMUNICATION FOR BUSINESS) — 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 1
+รวมต้องผ่านก่อน 2 วิชา</t>
+        </is>
+      </c>
+      <c r="H695" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 75, 23, 244, 270, 22, 27, 28, 32</t>
+        </is>
+      </c>
+      <c r="I695" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (วิชาบังคับก่อนไล่หลายชั้น) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J695" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K695" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L695" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M695" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/BIT/BIT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N695" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O695" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="696" ht="14.25" customHeight="1" s="36">
+      <c r="A696" s="37" t="inlineStr">
+        <is>
+          <t>SH9</t>
+        </is>
+      </c>
+      <c r="B696" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C696" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D696" s="39" t="inlineStr">
+        <is>
+          <t>ปี 1 ภาคต้นกับภาคปลาย ภาคไหนเรียนหนักกว่า ต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E696" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F696" s="39" t="inlineStr">
+        <is>
+          <t>ภาค 1 18, ภาค 2 21</t>
+        </is>
+      </c>
+      <c r="G696" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 1 ภาคการศึกษาที่ 2 หนักกว่า (21 เทียบกับ 18 หน่วยกิต) ต่างกัน 3 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ DSBA 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 1 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 23)
+- ปีที่ 1 ภาคการศึกษาที่ 2: 21 หน่วยกิต (หน้า 24)</t>
+        </is>
+      </c>
+      <c r="H696" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 23, 24</t>
+        </is>
+      </c>
+      <c r="I696" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J696" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K696" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L696" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M696" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N696" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O696" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="697" ht="14.25" customHeight="1" s="36">
+      <c r="A697" s="37" t="inlineStr">
+        <is>
+          <t>SH10</t>
+        </is>
+      </c>
+      <c r="B697" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C697" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D697" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเรียนตามแผน ตลอดปีที่ 3 รวมสองเทอมได้กี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E697" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F697" s="39" t="inlineStr">
+        <is>
+          <t>18 + 18</t>
+        </is>
+      </c>
+      <c r="G697" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 3 ตามแผนปกติเรียนรวม 36 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ DSBA 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 3 ภาคการศึกษาที่ 1: 18 หน่วยกิต (หน้า 27)
+- ปีที่ 3 ภาคการศึกษาที่ 2: 18 หน่วยกิต (หน้า 28)</t>
+        </is>
+      </c>
+      <c r="H697" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 27, 28</t>
+        </is>
+      </c>
+      <c r="I697" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J697" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K697" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L697" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M697" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N697" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O697" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="698" ht="14.25" customHeight="1" s="36">
+      <c r="A698" s="37" t="inlineStr">
+        <is>
+          <t>SH11</t>
+        </is>
+      </c>
+      <c r="B698" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C698" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D698" s="39" t="inlineStr">
+        <is>
+          <t>การแสดงข้อมูลด้วยแผนภาพ บวก เครือข่ายและความมั่นคงทางไซเบอร์เบื่องต้น ได้หน่วยกิตรวมเท่าไร</t>
+        </is>
+      </c>
+      <c r="E698" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F698" s="39" t="inlineStr">
+        <is>
+          <t>3 + 3</t>
+        </is>
+      </c>
+      <c r="G698" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: รวม 6 หน่วยกิต (3 + 3)
+- 06026209 การแสดงข้อมูลด้วยแผนภาพ (DATA VISUALIZATION) — 3(2-2-5) | ปีที่ 2 ภาคการศึกษาที่ 2
+- 06026204 เครือข่ายและความมั่นคงทางไซเบอร์เบื้องต้น (INTRODUCTION TO NETWORKS AND CYBERSECURITY) — 3(3-0-6) | ปีที่ 2 ภาคการศึกษาที่ 2</t>
+        </is>
+      </c>
+      <c r="H698" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 26, 33, 68, 17, 18, 316, 322, 353</t>
+        </is>
+      </c>
+      <c r="I698" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J698" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K698" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L698" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M698" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/DSBA/DSBA_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N698" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O698" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="699" ht="14.25" customHeight="1" s="36">
+      <c r="A699" s="37" t="inlineStr">
+        <is>
+          <t>SH12</t>
+        </is>
+      </c>
+      <c r="B699" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C699" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D699" s="39" t="inlineStr">
+        <is>
+          <t>ปี 4 ภาคต้นกับภาคปลาย ภาคไหนเรียนหนักกว่า ต่างกันกี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E699" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F699" s="39" t="inlineStr">
+        <is>
+          <t>ภาค 1 15, ภาค 2 9</t>
+        </is>
+      </c>
+      <c r="G699" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ปีที่ 4 ภาคการศึกษาที่ 1 หนักกว่า (15 เทียบกับ 9 หน่วยกิต) ต่างกัน 6 หน่วยกิต
+หน่วยกิตต่อภาคตามแผนปกติของ IT 2565 (ปริญญาตรี) (บรรทัด 'รวม' ของแต่ละภาค รวมวิชาเลือกที่แผนกำหนดแล้ว):
+- ปีที่ 4 ภาคการศึกษาที่ 1: 15 หน่วยกิต (หน้า 37)
+- ปีที่ 4 ภาคการศึกษาที่ 2: 9 หน่วยกิต (หน้า 37)</t>
+        </is>
+      </c>
+      <c r="H699" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 37</t>
+        </is>
+      </c>
+      <c r="I699" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (เทียบภาค/ทั้งปี/สะสมตามแผน) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J699" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K699" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L699" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M699" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N699" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O699" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="700" ht="14.25" customHeight="1" s="36">
+      <c r="A700" s="37" t="inlineStr">
+        <is>
+          <t>SH13</t>
+        </is>
+      </c>
+      <c r="B700" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C700" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D700" s="39" t="inlineStr">
+        <is>
+          <t>ระบบคอมพิวเตอร์เบื้องต้น บวก วิศวกรรมความต้องการ ได้หน่วยกิตรวมเท่าไร</t>
+        </is>
+      </c>
+      <c r="E700" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F700" s="39" t="inlineStr">
+        <is>
+          <t>3 + 3</t>
+        </is>
+      </c>
+      <c r="G700" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: รวม 6 หน่วยกิต (3 + 3)
+- 06016411 ระบบคอมพิวเตอร์เบื้องต้น (INTRODUCTION TO COMPUTER SYSTEMS) — 3(2-2-5) | ปีที่ 1 ภาคการศึกษาที่ 1
+- 06016416 วิศวกรรมความต้องการ (REQUIREMENT ENGINEERING) — 3(3-0-6) | ปีที่ 3 ภาคการศึกษาที่ 1</t>
+        </is>
+      </c>
+      <c r="H700" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 84, 24, 25, 31, 35, 38, 328, 330</t>
+        </is>
+      </c>
+      <c r="I700" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมของสองวิชา) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J700" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K700" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L700" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M700" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N700" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O700" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="701" ht="14.25" customHeight="1" s="36">
+      <c r="A701" s="37" t="inlineStr">
+        <is>
+          <t>SH14</t>
+        </is>
+      </c>
+      <c r="B701" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 3: ยาก</t>
+        </is>
+      </c>
+      <c r="C701" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D701" s="39" t="inlineStr">
+        <is>
+          <t>ถ้าเลื่อนวิชาการพัฒนาเว็บฝั่งเซิร์ฟเวอร์ ไปเรียนปี 4 จะได้หรือเปล่า</t>
+        </is>
+      </c>
+      <c r="E701" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F701" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ตามแผนปี 3 ต้องผ่าน 06016408</t>
+        </is>
+      </c>
+      <c r="G701" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ได้ — ตามแผนวิชานี้อยู่ปีที่ 3 อยู่แล้ว (ต้องผ่านวิชาบังคับก่อนข้างต้นก่อน)
+วิชา 06016418 การพัฒนาเว็บฝั่งเซิร์ฟเวอร์ (SERVER-SIDE WEB DEVELOPMENT) — 3(2-2-5) หน่วยกิต
+ตามแผนการศึกษา: ปีที่ 3 ภาคการศึกษาที่ 1
+วิชาบังคับก่อน (ต้องสอบผ่านก่อนจึงจะลงได้):
+  - 06016408 การสร้างโปรแกรมเชิงวัตถุ (OBJECT-ORIENTED PROGRAMMING) — ปีที่ 1 ภาคการศึกษาที่ 2</t>
+        </is>
+      </c>
+      <c r="H701" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 331, 24, 25, 26, 32, 35, 39, 83</t>
+        </is>
+      </c>
+      <c r="I701" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (ปีตามแผน + วิชาบังคับก่อน → ลงได้/ไม่ได้) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J701" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="K701" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L701" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M701" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/IT/IT_academic_plan_no_coop.json)</t>
+        </is>
+      </c>
+      <c r="N701" s="39" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="O701" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="702" ht="14.25" customHeight="1" s="36">
+      <c r="A702" s="37" t="inlineStr">
+        <is>
+          <t>SC4</t>
+        </is>
+      </c>
+      <c r="B702" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C702" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D702" s="39" t="inlineStr">
+        <is>
+          <t>เกรดเฉลี่ยตอนจบ 3.49 ได้เกียรตินิยมอันดับไหน</t>
+        </is>
+      </c>
+      <c r="E702" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F702" s="39" t="inlineStr">
+        <is>
+          <t>อันดับ 2 (ไม่ถึง 3.50)</t>
+        </is>
+      </c>
+      <c r="G702" s="39" t="inlineStr">
+        <is>
+          <t>ปริญญาเกียรตินิยม — ข้อ 36 ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 88, 89
+(ข้อบังคับของสถาบัน ใช้กับทุกหลักสูตรปริญญาตรี)
+- เกียรตินิยมอันดับหนึ่งและเหรียญทอง: ค่าระดับคะแนนเฉลี่ยสะสมตามโครงสร้างหลักสูตรสูงสุดในกลุ่มผู้สำเร็จการศึกษาปีเดียวกันของหลักสูตร และค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.75 และต้องไม่เทียบโอนผลการเรียนจากสถาบันอื่น
+- เกียรตินิยมอันดับหนึ่ง: ค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.50
+- เกียรตินิยมอันดับสอง: ค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 3.25
+- กรณีโอนผลการเรียนจากสถาบันอื่น ทุกรายวิชาต้องได้ไม่ต่ำกว่า B หรือ S และต้องเรียนในหลักสูตรของสถาบันไม่น้อยกว่า 2 ใน 3 ของหน่วยกิตรวม
+- เงื่อนไขทั่วไป (ข้อ 36.1): เรียนไม่เกินระยะเวลาตามแผนการศึกษา · ไม่มีรายวิชาใดได้ F หรือ U · ไม่เคยเรียนซ้ำเพื่อเปลี่ยนเกรด · ไม่เคยลาพักเพราะไม่ลงทะเบียนตามกำหนด และไม่เคยถูกลงโทษทางวินัย</t>
+        </is>
+      </c>
+      <c r="H702" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 88, 89</t>
+        </is>
+      </c>
+      <c r="I702" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J702" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K702" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L702" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M702" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N702" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O702" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="703" ht="14.25" customHeight="1" s="36">
+      <c r="A703" s="37" t="inlineStr">
+        <is>
+          <t>SC5</t>
+        </is>
+      </c>
+      <c r="B703" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C703" s="39" t="inlineStr">
+        <is>
+          <t>DSBA</t>
+        </is>
+      </c>
+      <c r="D703" s="39" t="inlineStr">
+        <is>
+          <t>ปีสุดท้ายเหลือวิชาอีก 25 หน่วยกิต ลงเทอมเดียวให้จบได้ไหม</t>
+        </is>
+      </c>
+      <c r="E703" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F703" s="39" t="inlineStr">
+        <is>
+          <t>ได้ ข้อยกเว้นปีสุดท้ายไม่เกิน 27</t>
+        </is>
+      </c>
+      <c r="G703" s="39" t="inlineStr">
+        <is>
+          <t>ได้ — นักศึกษาชั้นปีสุดท้ายที่เหลือวิชาไม่ถึง 9 หน่วยกิตหรือต้องลงเกิน 22 หน่วยกิตเพื่อสำเร็จการศึกษา สามารถลงทะเบียนได้ไม่เกิน 27 หน่วยกิตในภาคการศึกษาปกติ (ข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี ภาคผนวก มคอ.2 AIT 2566 หน้า 82) โดยหลักสูตร DSBA 2565 มีหน่วยกิตรวม 132 หน่วยกิต และนักศึกษาปีสุดท้ายสามารถลงวิชาได้สูงสุด 27 หน่วยกิตในภาคเดียว หากจำเป็นต้องสำเร็จการศึกษา.</t>
+        </is>
+      </c>
+      <c r="H703" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 82</t>
+        </is>
+      </c>
+      <c r="I703" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) → Typhoon เรียบเรียง</t>
+        </is>
+      </c>
+      <c r="J703" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K703" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L703" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M703" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก ข้อบังคับ ป.ตรี (AIT 2566 ภาคผนวก หน้า 82, 87, 89))</t>
+        </is>
+      </c>
+      <c r="N703" s="39" t="inlineStr">
+        <is>
+          <t>2.44s</t>
+        </is>
+      </c>
+      <c r="O703" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="704" ht="14.25" customHeight="1" s="36">
+      <c r="A704" s="37" t="inlineStr">
+        <is>
+          <t>SC6</t>
+        </is>
+      </c>
+      <c r="B704" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C704" s="39" t="inlineStr">
+        <is>
+          <t>AIT</t>
+        </is>
+      </c>
+      <c r="D704" s="39" t="inlineStr">
+        <is>
+          <t>ติดโปรอยู่ ต้องดึงเกรดเฉลี่ยสะสมให้ได้เท่าไรถึงจะหลุดโปร</t>
+        </is>
+      </c>
+      <c r="E704" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F704" s="39" t="inlineStr">
+        <is>
+          <t>ไม่ต่ำกว่า 2.00</t>
+        </is>
+      </c>
+      <c r="G704" s="39" t="inlineStr">
+        <is>
+          <t>การภาคทัณฑ์ — ข้อ 31 ตามข้อบังคับ สจล. ว่าด้วยการศึกษาระดับปริญญาตรี (ภาคผนวกในเล่ม มคอ.2 AIT 2566) หน้า 87
+(ข้อบังคับของสถาบัน ใช้กับทุกหลักสูตรปริญญาตรี)
+- นักศึกษาที่ได้ค่าระดับคะแนนเฉลี่ยสะสมต่ำกว่า 2.00 ต้องถูกภาคทัณฑ์
+- จะพ้นภาคทัณฑ์เมื่อค่าระดับคะแนนเฉลี่ยสะสมไม่ต่ำกว่า 2.00 (นับรวมภาคการศึกษาพิเศษด้วย)
+- ถ้าระหว่างภาคทัณฑ์ได้ค่าระดับคะแนนเฉลี่ยประจำภาคถัดไปต่ำกว่า 2.00 จะพ้นสภาพนักศึกษา (ข้อ 43.10)</t>
+        </is>
+      </c>
+      <c r="H704" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 87</t>
+        </is>
+      </c>
+      <c r="I704" s="39" t="inlineStr">
+        <is>
+          <t>ข้อบังคับปริญญาตรี (ภาคผนวกเล่ม AIT 2566) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J704" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K704" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L704" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M704" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก ข้อบังคับ ป.ตรี (AIT 2566 ภาคผนวก หน้า 82, 87, 89))</t>
+        </is>
+      </c>
+      <c r="N704" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O704" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="705" ht="14.25" customHeight="1" s="36">
+      <c r="A705" s="37" t="inlineStr">
+        <is>
+          <t>SC7</t>
+        </is>
+      </c>
+      <c r="B705" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C705" s="39" t="inlineStr">
+        <is>
+          <t>BIT</t>
+        </is>
+      </c>
+      <c r="D705" s="39" t="inlineStr">
+        <is>
+          <t>มี 120 หน่วยกิต เกรดเฉลี่ยสะสม 2.10 สำเร็จการศึกษาได้แล้วหรือยัง</t>
+        </is>
+      </c>
+      <c r="E705" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F705" s="39" t="inlineStr">
+        <is>
+          <t>ยัง ขาด 6</t>
+        </is>
+      </c>
+      <c r="G705" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ยังจบไม่ได้
+หลักสูตร BIT 2565 (ปริญญาตรี) ต้องเรียนครบไม่น้อยกว่า 126 หน่วยกิต (หน้า 6)
+- หน่วยกิต: เก็บได้ 120 หน่วยกิต → ยังขาดอีก 6 หน่วยกิต (ต้องครบ 126)
+- เกรดเฉลี่ยสะสม 2.10 → ผ่านเกณฑ์ขั้นต่ำ 2.00 (ข้อ 34)
+- เงื่อนไขอื่นตามข้อ 34: สอบผ่านทุกรายวิชาตามโครงสร้างหลักสูตร และผ่านการสอบภาษาอังกฤษ (English Exit exam)</t>
+        </is>
+      </c>
+      <c r="H705" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 6, 88</t>
+        </is>
+      </c>
+      <c r="I705" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวม + เกรดขั้นต่ำ ข้อ 34) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J705" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K705" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L705" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M705" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N705" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O705" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="706" ht="14.25" customHeight="1" s="36">
+      <c r="A706" s="37" t="inlineStr">
+        <is>
+          <t>SC8</t>
+        </is>
+      </c>
+      <c r="B706" s="38" t="inlineStr">
+        <is>
+          <t>ระดับ 4: ท้าทาย</t>
+        </is>
+      </c>
+      <c r="C706" s="39" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D706" s="39" t="inlineStr">
+        <is>
+          <t>AIT กับ BIT หลักสูตรไหนเรียนน้อยกว่า น้อยกว่ากี่หน่วยกิต</t>
+        </is>
+      </c>
+      <c r="E706" s="39" t="inlineStr">
+        <is>
+          <t>ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย) — ชุดที่ระบบไม่เคยเห็น รอบ 9 (ยาก/ท้าทาย)</t>
+        </is>
+      </c>
+      <c r="F706" s="39" t="inlineStr">
+        <is>
+          <t>AIT 120 น้อยกว่า BIT 126 อยู่ 6</t>
+        </is>
+      </c>
+      <c r="G706" s="39" t="inlineStr">
+        <is>
+          <t>คำตอบ: ต่างกัน 6 หน่วยกิต (BIT 2565 (ปริญญาตรี) มากกว่า AIT 2566 (ปริญญาตรี))
+- AIT 2566 (ปริญญาตรี): ไม่น้อยกว่า 120 หน่วยกิต (หน้า 5)
+- BIT 2565 (ปริญญาตรี): ไม่น้อยกว่า 126 หน่วยกิต (หน้า 6)</t>
+        </is>
+      </c>
+      <c r="H706" s="39" t="inlineStr">
+        <is>
+          <t>หน้า 5, 6</t>
+        </is>
+      </c>
+      <c r="I706" s="39" t="inlineStr">
+        <is>
+          <t>Multi-hop SQL (หน่วยกิตรวมข้ามหลักสูตร) — ไม่ผ่าน LLM</t>
+        </is>
+      </c>
+      <c r="J706" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K706" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L706" s="41" t="inlineStr">
+        <is>
+          <t>ถูกครบ</t>
+        </is>
+      </c>
+      <c r="M706" s="39" t="inlineStr">
+        <is>
+          <t>ตรวจอัตโนมัติ: คำตอบมีค่าตามเฉลยครบ (เฉลยจาก teacher_gt/rules_ground_truth.json)</t>
+        </is>
+      </c>
+      <c r="N706" s="39" t="inlineStr">
+        <is>
+          <t>0.00s</t>
+        </is>
+      </c>
+      <c r="O706" s="41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
     <row r="707" ht="14.25" customHeight="1" s="36"/>
     <row r="708" ht="14.25" customHeight="1" s="36"/>
     <row r="709" ht="14.25" customHeight="1" s="36"/>

</xml_diff>